<commit_message>
fix(helper): point pool 1st/2nd matchWinners at ranking formula cells (mp-c5c)
The elimination bracket's CONCATENATE formulas read the resolved
player names for "Pool X-1st"/"-2nd"/... from cells stored in
matchWinners. printSinglePool was assigning those cells AFTER
advancing poolRow past the ranking block, so the references landed
on empty rows below the Ranking section — the bracket then displayed
"Pool A-1st " with no name. Bug was most visible with a single
pool of 8 players on a single shiaijo but affected every pool.

Capture the ranking-formula row directly and store that as the
matchWinners cell. Add a regression test that exercises sizes 3,
4, 6, 8 and asserts the cell points at an INDEX(...MATCH(N,...))
formula.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pools-example-large-max-size.xlsx
+++ b/pools-example-large-max-size.xlsx
@@ -3221,7 +3221,7 @@
         <f>"2. " &amp; data!$B$51</f>
       </c>
       <c r="E6" s="23" t="str">
-        <f>CONCATENATE("Pool B-1st ",'Pool Matches'!G35)</f>
+        <f>CONCATENATE("Pool B-1st ",'Pool Matches'!G32)</f>
       </c>
     </row>
     <row r="7">
@@ -3242,7 +3242,7 @@
         <f>'data'!$A$55</f>
       </c>
       <c r="C9" s="23" t="str">
-        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G19)</f>
+        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G16)</f>
       </c>
       <c r="G9" s="20"/>
       <c r="H9" s="22"/>
@@ -3265,7 +3265,7 @@
         <f>"2. " &amp; data!$B$54</f>
       </c>
       <c r="C11" s="23" t="str">
-        <f>CONCATENATE("Pool C-2nd ",'Pool Matches'!G53)</f>
+        <f>CONCATENATE("Pool C-2nd ",'Pool Matches'!G50)</f>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="20"/>
@@ -3282,7 +3282,7 @@
     <row r="13">
       <c r="A13" s="22"/>
       <c r="C13" s="23" t="str">
-        <f>CONCATENATE("Pool D-1st ",'Pool Matches'!G69)</f>
+        <f>CONCATENATE("Pool D-1st ",'Pool Matches'!G66)</f>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="22"/>
@@ -3304,7 +3304,7 @@
         <f>"1. " &amp; data!$B$56</f>
       </c>
       <c r="C15" s="23" t="str">
-        <f>CONCATENATE("Pool E-2nd ",'Pool Matches'!G87)</f>
+        <f>CONCATENATE("Pool E-2nd ",'Pool Matches'!G84)</f>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="20"/>
@@ -3329,7 +3329,7 @@
         <f>"3. " &amp; data!$B$58</f>
       </c>
       <c r="C17" s="23" t="str">
-        <f>CONCATENATE("Pool F-1st ",'Pool Matches'!G103)</f>
+        <f>CONCATENATE("Pool F-1st ",'Pool Matches'!G100)</f>
       </c>
       <c r="G17" s="20"/>
       <c r="K17" s="20"/>
@@ -3349,7 +3349,7 @@
         <f>'data'!$A$61</f>
       </c>
       <c r="C19" s="23" t="str">
-        <f>CONCATENATE("Pool G-2nd ",'Pool Matches'!G121)</f>
+        <f>CONCATENATE("Pool G-2nd ",'Pool Matches'!G118)</f>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="20"/>
@@ -3368,7 +3368,7 @@
         <f>"2. " &amp; data!$B$60</f>
       </c>
       <c r="C21" s="23" t="str">
-        <f>CONCATENATE("Pool H-1st ",'Pool Matches'!G137)</f>
+        <f>CONCATENATE("Pool H-1st ",'Pool Matches'!G134)</f>
       </c>
       <c r="K21" s="20"/>
     </row>
@@ -3385,7 +3385,7 @@
     <row r="23">
       <c r="A23" s="22"/>
       <c r="C23" s="23" t="str">
-        <f>CONCATENATE("Pool I-2nd ",'Pool Matches'!G155)</f>
+        <f>CONCATENATE("Pool I-2nd ",'Pool Matches'!G152)</f>
       </c>
       <c r="D23" s="15"/>
       <c r="E23" s="20"/>
@@ -3407,7 +3407,7 @@
         <f>"1. " &amp; data!$B$62</f>
       </c>
       <c r="C25" s="23" t="str">
-        <f>CONCATENATE("Pool J-1st ",'Pool Matches'!G171)</f>
+        <f>CONCATENATE("Pool J-1st ",'Pool Matches'!G168)</f>
       </c>
       <c r="G25" s="20"/>
       <c r="H25" s="22"/>
@@ -3432,7 +3432,7 @@
         <f>"3. " &amp; data!$B$64</f>
       </c>
       <c r="C27" s="23" t="str">
-        <f>CONCATENATE("Pool K-2nd ",'Pool Matches'!G189)</f>
+        <f>CONCATENATE("Pool K-2nd ",'Pool Matches'!G186)</f>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="20"/>
@@ -3452,7 +3452,7 @@
         <f>'data'!$A$67</f>
       </c>
       <c r="C29" s="23" t="str">
-        <f>CONCATENATE("Pool L-1st ",'Pool Matches'!G205)</f>
+        <f>CONCATENATE("Pool L-1st ",'Pool Matches'!G202)</f>
       </c>
       <c r="I29" s="20"/>
     </row>
@@ -3471,7 +3471,7 @@
         <f>"2. " &amp; data!$B$66</f>
       </c>
       <c r="C31" s="23" t="str">
-        <f>CONCATENATE("Pool M-2nd ",'Pool Matches'!G223)</f>
+        <f>CONCATENATE("Pool M-2nd ",'Pool Matches'!G220)</f>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="20"/>
@@ -3492,7 +3492,7 @@
     <row r="33">
       <c r="A33" s="22"/>
       <c r="C33" s="23" t="str">
-        <f>CONCATENATE("Pool N-1st ",'Pool Matches'!G239)</f>
+        <f>CONCATENATE("Pool N-1st ",'Pool Matches'!G236)</f>
       </c>
       <c r="G33" s="20"/>
     </row>
@@ -3512,7 +3512,7 @@
         <f>"1. " &amp; data!$B$68</f>
       </c>
       <c r="C35" s="23" t="str">
-        <f>CONCATENATE("Pool O-2nd ",'Pool Matches'!G257)</f>
+        <f>CONCATENATE("Pool O-2nd ",'Pool Matches'!G254)</f>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="20"/>
@@ -3602,7 +3602,7 @@
         <f>"1. " &amp; data!$B$74</f>
       </c>
       <c r="C5" s="23" t="str">
-        <f>CONCATENATE("Pool P-1st ",'Pool Matches'!G269)</f>
+        <f>CONCATENATE("Pool P-1st ",'Pool Matches'!G267)</f>
       </c>
     </row>
     <row r="6">
@@ -3619,7 +3619,7 @@
         <f>"3. " &amp; data!$B$76</f>
       </c>
       <c r="C7" s="23" t="str">
-        <f>CONCATENATE("Pool Q-2nd ",'Pool Matches'!O19)</f>
+        <f>CONCATENATE("Pool Q-2nd ",'Pool Matches'!O16)</f>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="20"/>
@@ -3637,7 +3637,7 @@
         <f>'data'!$A$79</f>
       </c>
       <c r="C9" s="23" t="str">
-        <f>CONCATENATE("Pool R-1st ",'Pool Matches'!O35)</f>
+        <f>CONCATENATE("Pool R-1st ",'Pool Matches'!O32)</f>
       </c>
       <c r="G9" s="20"/>
       <c r="H9" s="22"/>
@@ -3660,7 +3660,7 @@
         <f>"2. " &amp; data!$B$78</f>
       </c>
       <c r="C11" s="23" t="str">
-        <f>CONCATENATE("Pool S-2nd ",'Pool Matches'!O53)</f>
+        <f>CONCATENATE("Pool S-2nd ",'Pool Matches'!O50)</f>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="20"/>
@@ -3677,7 +3677,7 @@
     <row r="13">
       <c r="A13" s="22"/>
       <c r="C13" s="23" t="str">
-        <f>CONCATENATE("Pool T-1st ",'Pool Matches'!O69)</f>
+        <f>CONCATENATE("Pool T-1st ",'Pool Matches'!O66)</f>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="22"/>
@@ -3699,7 +3699,7 @@
         <f>"1. " &amp; data!$B$80</f>
       </c>
       <c r="C15" s="23" t="str">
-        <f>CONCATENATE("Pool U-2nd ",'Pool Matches'!O87)</f>
+        <f>CONCATENATE("Pool U-2nd ",'Pool Matches'!O84)</f>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="20"/>
@@ -3724,7 +3724,7 @@
         <f>"3. " &amp; data!$B$82</f>
       </c>
       <c r="C17" s="23" t="str">
-        <f>CONCATENATE("Pool V-1st ",'Pool Matches'!O103)</f>
+        <f>CONCATENATE("Pool V-1st ",'Pool Matches'!O100)</f>
       </c>
       <c r="G17" s="20"/>
       <c r="K17" s="20"/>
@@ -3744,7 +3744,7 @@
         <f>'data'!$A$85</f>
       </c>
       <c r="C19" s="23" t="str">
-        <f>CONCATENATE("Pool W-2nd ",'Pool Matches'!O121)</f>
+        <f>CONCATENATE("Pool W-2nd ",'Pool Matches'!O118)</f>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="20"/>
@@ -3763,7 +3763,7 @@
         <f>"2. " &amp; data!$B$84</f>
       </c>
       <c r="C21" s="23" t="str">
-        <f>CONCATENATE("Pool X-1st ",'Pool Matches'!O137)</f>
+        <f>CONCATENATE("Pool X-1st ",'Pool Matches'!O134)</f>
       </c>
       <c r="K21" s="20"/>
     </row>
@@ -3780,7 +3780,7 @@
     <row r="23">
       <c r="A23" s="22"/>
       <c r="C23" s="23" t="str">
-        <f>CONCATENATE("Pool Y-2nd ",'Pool Matches'!O155)</f>
+        <f>CONCATENATE("Pool Y-2nd ",'Pool Matches'!O152)</f>
       </c>
       <c r="D23" s="15"/>
       <c r="E23" s="20"/>
@@ -3802,7 +3802,7 @@
         <f>"1. " &amp; data!$B$86</f>
       </c>
       <c r="C25" s="23" t="str">
-        <f>CONCATENATE("Pool Z-1st ",'Pool Matches'!O171)</f>
+        <f>CONCATENATE("Pool Z-1st ",'Pool Matches'!O168)</f>
       </c>
       <c r="G25" s="20"/>
       <c r="H25" s="22"/>
@@ -3827,7 +3827,7 @@
         <f>"3. " &amp; data!$B$88</f>
       </c>
       <c r="C27" s="23" t="str">
-        <f>CONCATENATE("Pool AA-2nd ",'Pool Matches'!O189)</f>
+        <f>CONCATENATE("Pool AA-2nd ",'Pool Matches'!O186)</f>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="20"/>
@@ -3847,7 +3847,7 @@
         <f>'data'!$A$91</f>
       </c>
       <c r="C29" s="23" t="str">
-        <f>CONCATENATE("Pool BB-1st ",'Pool Matches'!O205)</f>
+        <f>CONCATENATE("Pool BB-1st ",'Pool Matches'!O202)</f>
       </c>
       <c r="I29" s="20"/>
     </row>
@@ -3866,7 +3866,7 @@
         <f>"2. " &amp; data!$B$90</f>
       </c>
       <c r="C31" s="23" t="str">
-        <f>CONCATENATE("Pool CC-2nd ",'Pool Matches'!O223)</f>
+        <f>CONCATENATE("Pool CC-2nd ",'Pool Matches'!O220)</f>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="20"/>
@@ -3887,7 +3887,7 @@
     <row r="33">
       <c r="A33" s="22"/>
       <c r="C33" s="23" t="str">
-        <f>CONCATENATE("Pool DD-1st ",'Pool Matches'!O239)</f>
+        <f>CONCATENATE("Pool DD-1st ",'Pool Matches'!O236)</f>
       </c>
       <c r="G33" s="20"/>
     </row>
@@ -3907,7 +3907,7 @@
         <f>"1. " &amp; data!$B$92</f>
       </c>
       <c r="C35" s="23" t="str">
-        <f>CONCATENATE("Pool EE-2nd ",'Pool Matches'!O255)</f>
+        <f>CONCATENATE("Pool EE-2nd ",'Pool Matches'!O253)</f>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="20"/>
@@ -12163,7 +12163,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="str">
-        <f>CONCATENATE("Pool B-2nd ",'Pool Matches'!G36)</f>
+        <f>CONCATENATE("Pool B-2nd ",'Pool Matches'!G33)</f>
       </c>
       <c r="B4" s="18"/>
       <c r="C4" s="18"/>
@@ -12171,10 +12171,10 @@
       <c r="E4" s="18"/>
       <c r="F4" s="18"/>
       <c r="G4" s="14" t="str">
-        <f>CONCATENATE("Pool C-1st ",'Pool Matches'!G52)</f>
+        <f>CONCATENATE("Pool C-1st ",'Pool Matches'!G49)</f>
       </c>
       <c r="I4" s="14" t="str">
-        <f>CONCATENATE("Pool C-2nd ",'Pool Matches'!G53)</f>
+        <f>CONCATENATE("Pool C-2nd ",'Pool Matches'!G50)</f>
       </c>
       <c r="J4" s="18"/>
       <c r="K4" s="18"/>
@@ -12182,7 +12182,7 @@
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
       <c r="O4" s="14" t="str">
-        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G19)</f>
+        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G16)</f>
       </c>
     </row>
     <row r="6">
@@ -12247,7 +12247,7 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="str">
-        <f>CONCATENATE("Pool D-2nd ",'Pool Matches'!G70)</f>
+        <f>CONCATENATE("Pool D-2nd ",'Pool Matches'!G67)</f>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="18"/>
@@ -12255,10 +12255,10 @@
       <c r="E12" s="18"/>
       <c r="F12" s="18"/>
       <c r="G12" s="14" t="str">
-        <f>CONCATENATE("Pool E-1st ",'Pool Matches'!G86)</f>
+        <f>CONCATENATE("Pool E-1st ",'Pool Matches'!G83)</f>
       </c>
       <c r="I12" s="14" t="str">
-        <f>CONCATENATE("Pool E-2nd ",'Pool Matches'!G87)</f>
+        <f>CONCATENATE("Pool E-2nd ",'Pool Matches'!G84)</f>
       </c>
       <c r="J12" s="18"/>
       <c r="K12" s="18"/>
@@ -12266,7 +12266,7 @@
       <c r="M12" s="18"/>
       <c r="N12" s="18"/>
       <c r="O12" s="14" t="str">
-        <f>CONCATENATE("Pool D-1st ",'Pool Matches'!G69)</f>
+        <f>CONCATENATE("Pool D-1st ",'Pool Matches'!G66)</f>
       </c>
     </row>
     <row r="14">
@@ -12331,7 +12331,7 @@
     </row>
     <row r="20">
       <c r="A20" s="14" t="str">
-        <f>CONCATENATE("Pool F-2nd ",'Pool Matches'!G104)</f>
+        <f>CONCATENATE("Pool F-2nd ",'Pool Matches'!G101)</f>
       </c>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
@@ -12339,10 +12339,10 @@
       <c r="E20" s="18"/>
       <c r="F20" s="18"/>
       <c r="G20" s="14" t="str">
-        <f>CONCATENATE("Pool G-1st ",'Pool Matches'!G120)</f>
+        <f>CONCATENATE("Pool G-1st ",'Pool Matches'!G117)</f>
       </c>
       <c r="I20" s="14" t="str">
-        <f>CONCATENATE("Pool G-2nd ",'Pool Matches'!G121)</f>
+        <f>CONCATENATE("Pool G-2nd ",'Pool Matches'!G118)</f>
       </c>
       <c r="J20" s="18"/>
       <c r="K20" s="18"/>
@@ -12350,7 +12350,7 @@
       <c r="M20" s="18"/>
       <c r="N20" s="18"/>
       <c r="O20" s="14" t="str">
-        <f>CONCATENATE("Pool F-1st ",'Pool Matches'!G103)</f>
+        <f>CONCATENATE("Pool F-1st ",'Pool Matches'!G100)</f>
       </c>
     </row>
     <row r="22">
@@ -12415,7 +12415,7 @@
     </row>
     <row r="28">
       <c r="A28" s="14" t="str">
-        <f>CONCATENATE("Pool H-2nd ",'Pool Matches'!G138)</f>
+        <f>CONCATENATE("Pool H-2nd ",'Pool Matches'!G135)</f>
       </c>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -12423,10 +12423,10 @@
       <c r="E28" s="18"/>
       <c r="F28" s="18"/>
       <c r="G28" s="14" t="str">
-        <f>CONCATENATE("Pool I-1st ",'Pool Matches'!G154)</f>
+        <f>CONCATENATE("Pool I-1st ",'Pool Matches'!G151)</f>
       </c>
       <c r="I28" s="14" t="str">
-        <f>CONCATENATE("Pool I-2nd ",'Pool Matches'!G155)</f>
+        <f>CONCATENATE("Pool I-2nd ",'Pool Matches'!G152)</f>
       </c>
       <c r="J28" s="18"/>
       <c r="K28" s="18"/>
@@ -12434,7 +12434,7 @@
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
       <c r="O28" s="14" t="str">
-        <f>CONCATENATE("Pool H-1st ",'Pool Matches'!G137)</f>
+        <f>CONCATENATE("Pool H-1st ",'Pool Matches'!G134)</f>
       </c>
     </row>
     <row r="30">
@@ -12499,7 +12499,7 @@
     </row>
     <row r="36">
       <c r="A36" s="14" t="str">
-        <f>CONCATENATE("Pool J-2nd ",'Pool Matches'!G172)</f>
+        <f>CONCATENATE("Pool J-2nd ",'Pool Matches'!G169)</f>
       </c>
       <c r="B36" s="18"/>
       <c r="C36" s="18"/>
@@ -12507,10 +12507,10 @@
       <c r="E36" s="18"/>
       <c r="F36" s="18"/>
       <c r="G36" s="14" t="str">
-        <f>CONCATENATE("Pool K-1st ",'Pool Matches'!G188)</f>
+        <f>CONCATENATE("Pool K-1st ",'Pool Matches'!G185)</f>
       </c>
       <c r="I36" s="14" t="str">
-        <f>CONCATENATE("Pool K-2nd ",'Pool Matches'!G189)</f>
+        <f>CONCATENATE("Pool K-2nd ",'Pool Matches'!G186)</f>
       </c>
       <c r="J36" s="18"/>
       <c r="K36" s="18"/>
@@ -12518,7 +12518,7 @@
       <c r="M36" s="18"/>
       <c r="N36" s="18"/>
       <c r="O36" s="14" t="str">
-        <f>CONCATENATE("Pool J-1st ",'Pool Matches'!G171)</f>
+        <f>CONCATENATE("Pool J-1st ",'Pool Matches'!G168)</f>
       </c>
     </row>
     <row r="38">
@@ -12583,7 +12583,7 @@
     </row>
     <row r="44">
       <c r="A44" s="14" t="str">
-        <f>CONCATENATE("Pool L-2nd ",'Pool Matches'!G206)</f>
+        <f>CONCATENATE("Pool L-2nd ",'Pool Matches'!G203)</f>
       </c>
       <c r="B44" s="18"/>
       <c r="C44" s="18"/>
@@ -12591,10 +12591,10 @@
       <c r="E44" s="18"/>
       <c r="F44" s="18"/>
       <c r="G44" s="14" t="str">
-        <f>CONCATENATE("Pool M-1st ",'Pool Matches'!G222)</f>
+        <f>CONCATENATE("Pool M-1st ",'Pool Matches'!G219)</f>
       </c>
       <c r="I44" s="14" t="str">
-        <f>CONCATENATE("Pool M-2nd ",'Pool Matches'!G223)</f>
+        <f>CONCATENATE("Pool M-2nd ",'Pool Matches'!G220)</f>
       </c>
       <c r="J44" s="18"/>
       <c r="K44" s="18"/>
@@ -12602,7 +12602,7 @@
       <c r="M44" s="18"/>
       <c r="N44" s="18"/>
       <c r="O44" s="14" t="str">
-        <f>CONCATENATE("Pool L-1st ",'Pool Matches'!G205)</f>
+        <f>CONCATENATE("Pool L-1st ",'Pool Matches'!G202)</f>
       </c>
     </row>
     <row r="46">
@@ -12667,7 +12667,7 @@
     </row>
     <row r="52">
       <c r="A52" s="14" t="str">
-        <f>CONCATENATE("Pool N-2nd ",'Pool Matches'!G240)</f>
+        <f>CONCATENATE("Pool N-2nd ",'Pool Matches'!G237)</f>
       </c>
       <c r="B52" s="18"/>
       <c r="C52" s="18"/>
@@ -12675,10 +12675,10 @@
       <c r="E52" s="18"/>
       <c r="F52" s="18"/>
       <c r="G52" s="14" t="str">
-        <f>CONCATENATE("Pool O-1st ",'Pool Matches'!G256)</f>
+        <f>CONCATENATE("Pool O-1st ",'Pool Matches'!G253)</f>
       </c>
       <c r="I52" s="14" t="str">
-        <f>CONCATENATE("Pool O-2nd ",'Pool Matches'!G257)</f>
+        <f>CONCATENATE("Pool O-2nd ",'Pool Matches'!G254)</f>
       </c>
       <c r="J52" s="18"/>
       <c r="K52" s="18"/>
@@ -12686,7 +12686,7 @@
       <c r="M52" s="18"/>
       <c r="N52" s="18"/>
       <c r="O52" s="14" t="str">
-        <f>CONCATENATE("Pool N-1st ",'Pool Matches'!G239)</f>
+        <f>CONCATENATE("Pool N-1st ",'Pool Matches'!G236)</f>
       </c>
     </row>
     <row r="54">
@@ -12751,7 +12751,7 @@
     </row>
     <row r="60">
       <c r="A60" s="14" t="str">
-        <f>CONCATENATE("Pool P-2nd ",'Pool Matches'!G270)</f>
+        <f>CONCATENATE("Pool P-2nd ",'Pool Matches'!G268)</f>
       </c>
       <c r="B60" s="18"/>
       <c r="C60" s="18"/>
@@ -12759,10 +12759,10 @@
       <c r="E60" s="18"/>
       <c r="F60" s="18"/>
       <c r="G60" s="14" t="str">
-        <f>CONCATENATE("Pool Q-1st ",'Pool Matches'!O18)</f>
+        <f>CONCATENATE("Pool Q-1st ",'Pool Matches'!O15)</f>
       </c>
       <c r="I60" s="14" t="str">
-        <f>CONCATENATE("Pool Q-2nd ",'Pool Matches'!O19)</f>
+        <f>CONCATENATE("Pool Q-2nd ",'Pool Matches'!O16)</f>
       </c>
       <c r="J60" s="18"/>
       <c r="K60" s="18"/>
@@ -12770,7 +12770,7 @@
       <c r="M60" s="18"/>
       <c r="N60" s="18"/>
       <c r="O60" s="14" t="str">
-        <f>CONCATENATE("Pool P-1st ",'Pool Matches'!G269)</f>
+        <f>CONCATENATE("Pool P-1st ",'Pool Matches'!G267)</f>
       </c>
     </row>
     <row r="62">
@@ -12835,7 +12835,7 @@
     </row>
     <row r="68">
       <c r="A68" s="14" t="str">
-        <f>CONCATENATE("Pool R-2nd ",'Pool Matches'!O36)</f>
+        <f>CONCATENATE("Pool R-2nd ",'Pool Matches'!O33)</f>
       </c>
       <c r="B68" s="18"/>
       <c r="C68" s="18"/>
@@ -12843,10 +12843,10 @@
       <c r="E68" s="18"/>
       <c r="F68" s="18"/>
       <c r="G68" s="14" t="str">
-        <f>CONCATENATE("Pool S-1st ",'Pool Matches'!O52)</f>
+        <f>CONCATENATE("Pool S-1st ",'Pool Matches'!O49)</f>
       </c>
       <c r="I68" s="14" t="str">
-        <f>CONCATENATE("Pool S-2nd ",'Pool Matches'!O53)</f>
+        <f>CONCATENATE("Pool S-2nd ",'Pool Matches'!O50)</f>
       </c>
       <c r="J68" s="18"/>
       <c r="K68" s="18"/>
@@ -12854,7 +12854,7 @@
       <c r="M68" s="18"/>
       <c r="N68" s="18"/>
       <c r="O68" s="14" t="str">
-        <f>CONCATENATE("Pool R-1st ",'Pool Matches'!O35)</f>
+        <f>CONCATENATE("Pool R-1st ",'Pool Matches'!O32)</f>
       </c>
     </row>
     <row r="70">
@@ -12919,7 +12919,7 @@
     </row>
     <row r="76">
       <c r="A76" s="14" t="str">
-        <f>CONCATENATE("Pool T-2nd ",'Pool Matches'!O70)</f>
+        <f>CONCATENATE("Pool T-2nd ",'Pool Matches'!O67)</f>
       </c>
       <c r="B76" s="18"/>
       <c r="C76" s="18"/>
@@ -12927,10 +12927,10 @@
       <c r="E76" s="18"/>
       <c r="F76" s="18"/>
       <c r="G76" s="14" t="str">
-        <f>CONCATENATE("Pool U-1st ",'Pool Matches'!O86)</f>
+        <f>CONCATENATE("Pool U-1st ",'Pool Matches'!O83)</f>
       </c>
       <c r="I76" s="14" t="str">
-        <f>CONCATENATE("Pool U-2nd ",'Pool Matches'!O87)</f>
+        <f>CONCATENATE("Pool U-2nd ",'Pool Matches'!O84)</f>
       </c>
       <c r="J76" s="18"/>
       <c r="K76" s="18"/>
@@ -12938,7 +12938,7 @@
       <c r="M76" s="18"/>
       <c r="N76" s="18"/>
       <c r="O76" s="14" t="str">
-        <f>CONCATENATE("Pool T-1st ",'Pool Matches'!O69)</f>
+        <f>CONCATENATE("Pool T-1st ",'Pool Matches'!O66)</f>
       </c>
     </row>
     <row r="78">
@@ -13003,7 +13003,7 @@
     </row>
     <row r="84">
       <c r="A84" s="14" t="str">
-        <f>CONCATENATE("Pool V-2nd ",'Pool Matches'!O104)</f>
+        <f>CONCATENATE("Pool V-2nd ",'Pool Matches'!O101)</f>
       </c>
       <c r="B84" s="18"/>
       <c r="C84" s="18"/>
@@ -13011,10 +13011,10 @@
       <c r="E84" s="18"/>
       <c r="F84" s="18"/>
       <c r="G84" s="14" t="str">
-        <f>CONCATENATE("Pool W-1st ",'Pool Matches'!O120)</f>
+        <f>CONCATENATE("Pool W-1st ",'Pool Matches'!O117)</f>
       </c>
       <c r="I84" s="14" t="str">
-        <f>CONCATENATE("Pool W-2nd ",'Pool Matches'!O121)</f>
+        <f>CONCATENATE("Pool W-2nd ",'Pool Matches'!O118)</f>
       </c>
       <c r="J84" s="18"/>
       <c r="K84" s="18"/>
@@ -13022,7 +13022,7 @@
       <c r="M84" s="18"/>
       <c r="N84" s="18"/>
       <c r="O84" s="14" t="str">
-        <f>CONCATENATE("Pool V-1st ",'Pool Matches'!O103)</f>
+        <f>CONCATENATE("Pool V-1st ",'Pool Matches'!O100)</f>
       </c>
     </row>
     <row r="86">
@@ -13087,7 +13087,7 @@
     </row>
     <row r="92">
       <c r="A92" s="14" t="str">
-        <f>CONCATENATE("Pool X-2nd ",'Pool Matches'!O138)</f>
+        <f>CONCATENATE("Pool X-2nd ",'Pool Matches'!O135)</f>
       </c>
       <c r="B92" s="18"/>
       <c r="C92" s="18"/>
@@ -13095,10 +13095,10 @@
       <c r="E92" s="18"/>
       <c r="F92" s="18"/>
       <c r="G92" s="14" t="str">
-        <f>CONCATENATE("Pool Y-1st ",'Pool Matches'!O154)</f>
+        <f>CONCATENATE("Pool Y-1st ",'Pool Matches'!O151)</f>
       </c>
       <c r="I92" s="14" t="str">
-        <f>CONCATENATE("Pool Y-2nd ",'Pool Matches'!O155)</f>
+        <f>CONCATENATE("Pool Y-2nd ",'Pool Matches'!O152)</f>
       </c>
       <c r="J92" s="18"/>
       <c r="K92" s="18"/>
@@ -13106,7 +13106,7 @@
       <c r="M92" s="18"/>
       <c r="N92" s="18"/>
       <c r="O92" s="14" t="str">
-        <f>CONCATENATE("Pool X-1st ",'Pool Matches'!O137)</f>
+        <f>CONCATENATE("Pool X-1st ",'Pool Matches'!O134)</f>
       </c>
     </row>
     <row r="94">
@@ -13171,7 +13171,7 @@
     </row>
     <row r="100">
       <c r="A100" s="14" t="str">
-        <f>CONCATENATE("Pool Z-2nd ",'Pool Matches'!O172)</f>
+        <f>CONCATENATE("Pool Z-2nd ",'Pool Matches'!O169)</f>
       </c>
       <c r="B100" s="18"/>
       <c r="C100" s="18"/>
@@ -13179,10 +13179,10 @@
       <c r="E100" s="18"/>
       <c r="F100" s="18"/>
       <c r="G100" s="14" t="str">
-        <f>CONCATENATE("Pool AA-1st ",'Pool Matches'!O188)</f>
+        <f>CONCATENATE("Pool AA-1st ",'Pool Matches'!O185)</f>
       </c>
       <c r="I100" s="14" t="str">
-        <f>CONCATENATE("Pool AA-2nd ",'Pool Matches'!O189)</f>
+        <f>CONCATENATE("Pool AA-2nd ",'Pool Matches'!O186)</f>
       </c>
       <c r="J100" s="18"/>
       <c r="K100" s="18"/>
@@ -13190,7 +13190,7 @@
       <c r="M100" s="18"/>
       <c r="N100" s="18"/>
       <c r="O100" s="14" t="str">
-        <f>CONCATENATE("Pool Z-1st ",'Pool Matches'!O171)</f>
+        <f>CONCATENATE("Pool Z-1st ",'Pool Matches'!O168)</f>
       </c>
     </row>
     <row r="102">
@@ -13255,7 +13255,7 @@
     </row>
     <row r="108">
       <c r="A108" s="14" t="str">
-        <f>CONCATENATE("Pool BB-2nd ",'Pool Matches'!O206)</f>
+        <f>CONCATENATE("Pool BB-2nd ",'Pool Matches'!O203)</f>
       </c>
       <c r="B108" s="18"/>
       <c r="C108" s="18"/>
@@ -13263,10 +13263,10 @@
       <c r="E108" s="18"/>
       <c r="F108" s="18"/>
       <c r="G108" s="14" t="str">
-        <f>CONCATENATE("Pool CC-1st ",'Pool Matches'!O222)</f>
+        <f>CONCATENATE("Pool CC-1st ",'Pool Matches'!O219)</f>
       </c>
       <c r="I108" s="14" t="str">
-        <f>CONCATENATE("Pool CC-2nd ",'Pool Matches'!O223)</f>
+        <f>CONCATENATE("Pool CC-2nd ",'Pool Matches'!O220)</f>
       </c>
       <c r="J108" s="18"/>
       <c r="K108" s="18"/>
@@ -13274,7 +13274,7 @@
       <c r="M108" s="18"/>
       <c r="N108" s="18"/>
       <c r="O108" s="14" t="str">
-        <f>CONCATENATE("Pool BB-1st ",'Pool Matches'!O205)</f>
+        <f>CONCATENATE("Pool BB-1st ",'Pool Matches'!O202)</f>
       </c>
     </row>
     <row r="110">
@@ -13339,7 +13339,7 @@
     </row>
     <row r="116">
       <c r="A116" s="14" t="str">
-        <f>CONCATENATE("Pool DD-2nd ",'Pool Matches'!O240)</f>
+        <f>CONCATENATE("Pool DD-2nd ",'Pool Matches'!O237)</f>
       </c>
       <c r="B116" s="18"/>
       <c r="C116" s="18"/>
@@ -13347,10 +13347,10 @@
       <c r="E116" s="18"/>
       <c r="F116" s="18"/>
       <c r="G116" s="14" t="str">
-        <f>CONCATENATE("Pool EE-1st ",'Pool Matches'!O254)</f>
+        <f>CONCATENATE("Pool EE-1st ",'Pool Matches'!O252)</f>
       </c>
       <c r="I116" s="14" t="str">
-        <f>CONCATENATE("Pool EE-2nd ",'Pool Matches'!O255)</f>
+        <f>CONCATENATE("Pool EE-2nd ",'Pool Matches'!O253)</f>
       </c>
       <c r="J116" s="18"/>
       <c r="K116" s="18"/>
@@ -13358,7 +13358,7 @@
       <c r="M116" s="18"/>
       <c r="N116" s="18"/>
       <c r="O116" s="14" t="str">
-        <f>CONCATENATE("Pool DD-1st ",'Pool Matches'!O239)</f>
+        <f>CONCATENATE("Pool DD-1st ",'Pool Matches'!O236)</f>
       </c>
     </row>
     <row r="118">
@@ -13431,7 +13431,7 @@
       <c r="E129" s="18"/>
       <c r="F129" s="18"/>
       <c r="G129" s="14" t="str">
-        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G18)</f>
+        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G15)</f>
       </c>
       <c r="I129" s="14" t="str">
         <f>CONCATENATE("M 16 ",O6)</f>
@@ -13442,7 +13442,7 @@
       <c r="M129" s="18"/>
       <c r="N129" s="18"/>
       <c r="O129" s="14" t="str">
-        <f>CONCATENATE("Pool B-1st ",'Pool Matches'!G35)</f>
+        <f>CONCATENATE("Pool B-1st ",'Pool Matches'!G32)</f>
       </c>
     </row>
     <row r="131">
@@ -14815,7 +14815,7 @@
         <f>"2. " &amp; data!$B$4</f>
       </c>
       <c r="E6" s="23" t="str">
-        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G18)</f>
+        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G15)</f>
       </c>
     </row>
     <row r="7">
@@ -14836,7 +14836,7 @@
         <f>'data'!$A$8</f>
       </c>
       <c r="C9" s="23" t="str">
-        <f>CONCATENATE("Pool C-1st ",'Pool Matches'!G52)</f>
+        <f>CONCATENATE("Pool C-1st ",'Pool Matches'!G49)</f>
       </c>
       <c r="G9" s="20"/>
       <c r="H9" s="22"/>
@@ -14859,7 +14859,7 @@
         <f>"2. " &amp; data!$B$7</f>
       </c>
       <c r="C11" s="23" t="str">
-        <f>CONCATENATE("Pool B-2nd ",'Pool Matches'!G36)</f>
+        <f>CONCATENATE("Pool B-2nd ",'Pool Matches'!G33)</f>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="20"/>
@@ -14876,7 +14876,7 @@
     <row r="13">
       <c r="A13" s="22"/>
       <c r="C13" s="23" t="str">
-        <f>CONCATENATE("Pool E-1st ",'Pool Matches'!G86)</f>
+        <f>CONCATENATE("Pool E-1st ",'Pool Matches'!G83)</f>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="22"/>
@@ -14898,7 +14898,7 @@
         <f>"1. " &amp; data!$B$9</f>
       </c>
       <c r="C15" s="23" t="str">
-        <f>CONCATENATE("Pool D-2nd ",'Pool Matches'!G70)</f>
+        <f>CONCATENATE("Pool D-2nd ",'Pool Matches'!G67)</f>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="20"/>
@@ -14923,7 +14923,7 @@
         <f>"3. " &amp; data!$B$11</f>
       </c>
       <c r="C17" s="23" t="str">
-        <f>CONCATENATE("Pool G-1st ",'Pool Matches'!G120)</f>
+        <f>CONCATENATE("Pool G-1st ",'Pool Matches'!G117)</f>
       </c>
       <c r="G17" s="20"/>
       <c r="K17" s="20"/>
@@ -14943,7 +14943,7 @@
         <f>'data'!$A$14</f>
       </c>
       <c r="C19" s="23" t="str">
-        <f>CONCATENATE("Pool F-2nd ",'Pool Matches'!G104)</f>
+        <f>CONCATENATE("Pool F-2nd ",'Pool Matches'!G101)</f>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="20"/>
@@ -14962,7 +14962,7 @@
         <f>"2. " &amp; data!$B$13</f>
       </c>
       <c r="C21" s="23" t="str">
-        <f>CONCATENATE("Pool I-1st ",'Pool Matches'!G154)</f>
+        <f>CONCATENATE("Pool I-1st ",'Pool Matches'!G151)</f>
       </c>
       <c r="K21" s="20"/>
     </row>
@@ -14979,7 +14979,7 @@
     <row r="23">
       <c r="A23" s="22"/>
       <c r="C23" s="23" t="str">
-        <f>CONCATENATE("Pool H-2nd ",'Pool Matches'!G138)</f>
+        <f>CONCATENATE("Pool H-2nd ",'Pool Matches'!G135)</f>
       </c>
       <c r="D23" s="15"/>
       <c r="E23" s="20"/>
@@ -15001,7 +15001,7 @@
         <f>"1. " &amp; data!$B$15</f>
       </c>
       <c r="C25" s="23" t="str">
-        <f>CONCATENATE("Pool K-1st ",'Pool Matches'!G188)</f>
+        <f>CONCATENATE("Pool K-1st ",'Pool Matches'!G185)</f>
       </c>
       <c r="G25" s="20"/>
       <c r="H25" s="22"/>
@@ -15026,7 +15026,7 @@
         <f>"3. " &amp; data!$B$17</f>
       </c>
       <c r="C27" s="23" t="str">
-        <f>CONCATENATE("Pool J-2nd ",'Pool Matches'!G172)</f>
+        <f>CONCATENATE("Pool J-2nd ",'Pool Matches'!G169)</f>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="20"/>
@@ -15046,7 +15046,7 @@
         <f>'data'!$A$20</f>
       </c>
       <c r="C29" s="23" t="str">
-        <f>CONCATENATE("Pool M-1st ",'Pool Matches'!G222)</f>
+        <f>CONCATENATE("Pool M-1st ",'Pool Matches'!G219)</f>
       </c>
       <c r="I29" s="20"/>
     </row>
@@ -15065,7 +15065,7 @@
         <f>"2. " &amp; data!$B$19</f>
       </c>
       <c r="C31" s="23" t="str">
-        <f>CONCATENATE("Pool L-2nd ",'Pool Matches'!G206)</f>
+        <f>CONCATENATE("Pool L-2nd ",'Pool Matches'!G203)</f>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="20"/>
@@ -15086,7 +15086,7 @@
     <row r="33">
       <c r="A33" s="22"/>
       <c r="C33" s="23" t="str">
-        <f>CONCATENATE("Pool O-1st ",'Pool Matches'!G256)</f>
+        <f>CONCATENATE("Pool O-1st ",'Pool Matches'!G253)</f>
       </c>
       <c r="G33" s="20"/>
     </row>
@@ -15106,7 +15106,7 @@
         <f>"1. " &amp; data!$B$21</f>
       </c>
       <c r="C35" s="23" t="str">
-        <f>CONCATENATE("Pool N-2nd ",'Pool Matches'!G240)</f>
+        <f>CONCATENATE("Pool N-2nd ",'Pool Matches'!G237)</f>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="20"/>
@@ -15196,7 +15196,7 @@
         <f>"1. " &amp; data!$B$27</f>
       </c>
       <c r="C5" s="23" t="str">
-        <f>CONCATENATE("Pool Q-1st ",'Pool Matches'!O18)</f>
+        <f>CONCATENATE("Pool Q-1st ",'Pool Matches'!O15)</f>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <f>"3. " &amp; data!$B$29</f>
       </c>
       <c r="C7" s="23" t="str">
-        <f>CONCATENATE("Pool P-2nd ",'Pool Matches'!G270)</f>
+        <f>CONCATENATE("Pool P-2nd ",'Pool Matches'!G268)</f>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="20"/>
@@ -15231,7 +15231,7 @@
         <f>'data'!$A$32</f>
       </c>
       <c r="C9" s="23" t="str">
-        <f>CONCATENATE("Pool S-1st ",'Pool Matches'!O52)</f>
+        <f>CONCATENATE("Pool S-1st ",'Pool Matches'!O49)</f>
       </c>
       <c r="G9" s="20"/>
       <c r="H9" s="22"/>
@@ -15254,7 +15254,7 @@
         <f>"2. " &amp; data!$B$31</f>
       </c>
       <c r="C11" s="23" t="str">
-        <f>CONCATENATE("Pool R-2nd ",'Pool Matches'!O36)</f>
+        <f>CONCATENATE("Pool R-2nd ",'Pool Matches'!O33)</f>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="20"/>
@@ -15271,7 +15271,7 @@
     <row r="13">
       <c r="A13" s="22"/>
       <c r="C13" s="23" t="str">
-        <f>CONCATENATE("Pool U-1st ",'Pool Matches'!O86)</f>
+        <f>CONCATENATE("Pool U-1st ",'Pool Matches'!O83)</f>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="22"/>
@@ -15293,7 +15293,7 @@
         <f>"1. " &amp; data!$B$33</f>
       </c>
       <c r="C15" s="23" t="str">
-        <f>CONCATENATE("Pool T-2nd ",'Pool Matches'!O70)</f>
+        <f>CONCATENATE("Pool T-2nd ",'Pool Matches'!O67)</f>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="20"/>
@@ -15318,7 +15318,7 @@
         <f>"3. " &amp; data!$B$35</f>
       </c>
       <c r="C17" s="23" t="str">
-        <f>CONCATENATE("Pool W-1st ",'Pool Matches'!O120)</f>
+        <f>CONCATENATE("Pool W-1st ",'Pool Matches'!O117)</f>
       </c>
       <c r="G17" s="20"/>
       <c r="K17" s="20"/>
@@ -15338,7 +15338,7 @@
         <f>'data'!$A$38</f>
       </c>
       <c r="C19" s="23" t="str">
-        <f>CONCATENATE("Pool V-2nd ",'Pool Matches'!O104)</f>
+        <f>CONCATENATE("Pool V-2nd ",'Pool Matches'!O101)</f>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="20"/>
@@ -15357,7 +15357,7 @@
         <f>"2. " &amp; data!$B$37</f>
       </c>
       <c r="C21" s="23" t="str">
-        <f>CONCATENATE("Pool Y-1st ",'Pool Matches'!O154)</f>
+        <f>CONCATENATE("Pool Y-1st ",'Pool Matches'!O151)</f>
       </c>
       <c r="K21" s="20"/>
     </row>
@@ -15374,7 +15374,7 @@
     <row r="23">
       <c r="A23" s="22"/>
       <c r="C23" s="23" t="str">
-        <f>CONCATENATE("Pool X-2nd ",'Pool Matches'!O138)</f>
+        <f>CONCATENATE("Pool X-2nd ",'Pool Matches'!O135)</f>
       </c>
       <c r="D23" s="15"/>
       <c r="E23" s="20"/>
@@ -15396,7 +15396,7 @@
         <f>"1. " &amp; data!$B$39</f>
       </c>
       <c r="C25" s="23" t="str">
-        <f>CONCATENATE("Pool AA-1st ",'Pool Matches'!O188)</f>
+        <f>CONCATENATE("Pool AA-1st ",'Pool Matches'!O185)</f>
       </c>
       <c r="G25" s="20"/>
       <c r="H25" s="22"/>
@@ -15421,7 +15421,7 @@
         <f>"3. " &amp; data!$B$41</f>
       </c>
       <c r="C27" s="23" t="str">
-        <f>CONCATENATE("Pool Z-2nd ",'Pool Matches'!O172)</f>
+        <f>CONCATENATE("Pool Z-2nd ",'Pool Matches'!O169)</f>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="20"/>
@@ -15441,7 +15441,7 @@
         <f>'data'!$A$44</f>
       </c>
       <c r="C29" s="23" t="str">
-        <f>CONCATENATE("Pool CC-1st ",'Pool Matches'!O222)</f>
+        <f>CONCATENATE("Pool CC-1st ",'Pool Matches'!O219)</f>
       </c>
       <c r="I29" s="20"/>
     </row>
@@ -15460,7 +15460,7 @@
         <f>"2. " &amp; data!$B$43</f>
       </c>
       <c r="C31" s="23" t="str">
-        <f>CONCATENATE("Pool BB-2nd ",'Pool Matches'!O206)</f>
+        <f>CONCATENATE("Pool BB-2nd ",'Pool Matches'!O203)</f>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="20"/>
@@ -15481,7 +15481,7 @@
     <row r="33">
       <c r="A33" s="22"/>
       <c r="C33" s="23" t="str">
-        <f>CONCATENATE("Pool EE-1st ",'Pool Matches'!O254)</f>
+        <f>CONCATENATE("Pool EE-1st ",'Pool Matches'!O252)</f>
       </c>
       <c r="G33" s="20"/>
     </row>
@@ -15501,7 +15501,7 @@
         <f>"1. " &amp; data!$B$45</f>
       </c>
       <c r="C35" s="23" t="str">
-        <f>CONCATENATE("Pool DD-2nd ",'Pool Matches'!O240)</f>
+        <f>CONCATENATE("Pool DD-2nd ",'Pool Matches'!O237)</f>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="20"/>

</xml_diff>

<commit_message>
fix(helper): drop leading '=' from hierarchical-score formulas (mp-x7h)
The two scoreFormula strings in printPoolResultsTable helpers each had a
literal '=' at the start. excelize stored that '=' verbatim inside the
OOXML <f> element body, e.g.:

  <f>=(B34*1000000)-(C34*10000)+(D34*100)+(E34*1)-(F34*0.01)</f>

The spec says <f> holds the formula body only; the leading '=' is a UI
convention, not part of the formula. Excel is lenient and evaluates the
expression anyway, but Google Sheets and Apple Numbers reject it and
either produce #ERROR! or leave the cell blank. That broke the entire
Pool Results / Rank / Ranking chain whenever the workbook was opened
outside Excel.

Drop the prefix and add a regression assertion in the round-robin pool-
of-8 end-to-end test that scans every <f> element across every sheet
and fails if any starts with '='.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pools-example-large-max-size.xlsx
+++ b/pools-example-large-max-size.xlsx
@@ -6776,10 +6776,10 @@
         <f>RANK(AC9,$AC$9:$AC$11)+COUNTIF($AC$8:AC8,AC9)</f>
       </c>
       <c r="U9" t="str">
-        <f>=(B9*1000000)-(C9*10000)+(D9*100)+(E9*1)-(F9*0.01)</f>
+        <f>(B9*1000000)-(C9*10000)+(D9*100)+(E9*1)-(F9*0.01)</f>
       </c>
       <c r="AC9" t="str">
-        <f>=(J9*1000000)-(K9*10000)+(L9*100)+(M9*1)-(N9*0.01)</f>
+        <f>(J9*1000000)-(K9*10000)+(L9*100)+(M9*1)-(N9*0.01)</f>
       </c>
     </row>
     <row r="10">
@@ -6826,10 +6826,10 @@
         <f>RANK(AC10,$AC$9:$AC$11)+COUNTIF($AC$8:AC9,AC10)</f>
       </c>
       <c r="U10" t="str">
-        <f>=(B10*1000000)-(C10*10000)+(D10*100)+(E10*1)-(F10*0.01)</f>
+        <f>(B10*1000000)-(C10*10000)+(D10*100)+(E10*1)-(F10*0.01)</f>
       </c>
       <c r="AC10" t="str">
-        <f>=(J10*1000000)-(K10*10000)+(L10*100)+(M10*1)-(N10*0.01)</f>
+        <f>(J10*1000000)-(K10*10000)+(L10*100)+(M10*1)-(N10*0.01)</f>
       </c>
     </row>
     <row r="11">
@@ -6876,10 +6876,10 @@
         <f>RANK(AC11,$AC$9:$AC$11)+COUNTIF($AC$8:AC10,AC11)</f>
       </c>
       <c r="U11" t="str">
-        <f>=(B11*1000000)-(C11*10000)+(D11*100)+(E11*1)-(F11*0.01)</f>
+        <f>(B11*1000000)-(C11*10000)+(D11*100)+(E11*1)-(F11*0.01)</f>
       </c>
       <c r="AC11" t="str">
-        <f>=(J11*1000000)-(K11*10000)+(L11*100)+(M11*1)-(N11*0.01)</f>
+        <f>(J11*1000000)-(K11*10000)+(L11*100)+(M11*1)-(N11*0.01)</f>
       </c>
     </row>
     <row r="14">
@@ -7134,10 +7134,10 @@
         <f>RANK(AC26,$AC$26:$AC$28)+COUNTIF($AC$25:AC25,AC26)</f>
       </c>
       <c r="U26" t="str">
-        <f>=(B26*1000000)-(C26*10000)+(D26*100)+(E26*1)-(F26*0.01)</f>
+        <f>(B26*1000000)-(C26*10000)+(D26*100)+(E26*1)-(F26*0.01)</f>
       </c>
       <c r="AC26" t="str">
-        <f>=(J26*1000000)-(K26*10000)+(L26*100)+(M26*1)-(N26*0.01)</f>
+        <f>(J26*1000000)-(K26*10000)+(L26*100)+(M26*1)-(N26*0.01)</f>
       </c>
     </row>
     <row r="27">
@@ -7184,10 +7184,10 @@
         <f>RANK(AC27,$AC$26:$AC$28)+COUNTIF($AC$25:AC26,AC27)</f>
       </c>
       <c r="U27" t="str">
-        <f>=(B27*1000000)-(C27*10000)+(D27*100)+(E27*1)-(F27*0.01)</f>
+        <f>(B27*1000000)-(C27*10000)+(D27*100)+(E27*1)-(F27*0.01)</f>
       </c>
       <c r="AC27" t="str">
-        <f>=(J27*1000000)-(K27*10000)+(L27*100)+(M27*1)-(N27*0.01)</f>
+        <f>(J27*1000000)-(K27*10000)+(L27*100)+(M27*1)-(N27*0.01)</f>
       </c>
     </row>
     <row r="28">
@@ -7234,10 +7234,10 @@
         <f>RANK(AC28,$AC$26:$AC$28)+COUNTIF($AC$25:AC27,AC28)</f>
       </c>
       <c r="U28" t="str">
-        <f>=(B28*1000000)-(C28*10000)+(D28*100)+(E28*1)-(F28*0.01)</f>
+        <f>(B28*1000000)-(C28*10000)+(D28*100)+(E28*1)-(F28*0.01)</f>
       </c>
       <c r="AC28" t="str">
-        <f>=(J28*1000000)-(K28*10000)+(L28*100)+(M28*1)-(N28*0.01)</f>
+        <f>(J28*1000000)-(K28*10000)+(L28*100)+(M28*1)-(N28*0.01)</f>
       </c>
     </row>
     <row r="31">
@@ -7492,10 +7492,10 @@
         <f>RANK(AC43,$AC$43:$AC$45)+COUNTIF($AC$42:AC42,AC43)</f>
       </c>
       <c r="U43" t="str">
-        <f>=(B43*1000000)-(C43*10000)+(D43*100)+(E43*1)-(F43*0.01)</f>
+        <f>(B43*1000000)-(C43*10000)+(D43*100)+(E43*1)-(F43*0.01)</f>
       </c>
       <c r="AC43" t="str">
-        <f>=(J43*1000000)-(K43*10000)+(L43*100)+(M43*1)-(N43*0.01)</f>
+        <f>(J43*1000000)-(K43*10000)+(L43*100)+(M43*1)-(N43*0.01)</f>
       </c>
     </row>
     <row r="44">
@@ -7542,10 +7542,10 @@
         <f>RANK(AC44,$AC$43:$AC$45)+COUNTIF($AC$42:AC43,AC44)</f>
       </c>
       <c r="U44" t="str">
-        <f>=(B44*1000000)-(C44*10000)+(D44*100)+(E44*1)-(F44*0.01)</f>
+        <f>(B44*1000000)-(C44*10000)+(D44*100)+(E44*1)-(F44*0.01)</f>
       </c>
       <c r="AC44" t="str">
-        <f>=(J44*1000000)-(K44*10000)+(L44*100)+(M44*1)-(N44*0.01)</f>
+        <f>(J44*1000000)-(K44*10000)+(L44*100)+(M44*1)-(N44*0.01)</f>
       </c>
     </row>
     <row r="45">
@@ -7592,10 +7592,10 @@
         <f>RANK(AC45,$AC$43:$AC$45)+COUNTIF($AC$42:AC44,AC45)</f>
       </c>
       <c r="U45" t="str">
-        <f>=(B45*1000000)-(C45*10000)+(D45*100)+(E45*1)-(F45*0.01)</f>
+        <f>(B45*1000000)-(C45*10000)+(D45*100)+(E45*1)-(F45*0.01)</f>
       </c>
       <c r="AC45" t="str">
-        <f>=(J45*1000000)-(K45*10000)+(L45*100)+(M45*1)-(N45*0.01)</f>
+        <f>(J45*1000000)-(K45*10000)+(L45*100)+(M45*1)-(N45*0.01)</f>
       </c>
     </row>
     <row r="48">
@@ -7850,10 +7850,10 @@
         <f>RANK(AC60,$AC$60:$AC$62)+COUNTIF($AC$59:AC59,AC60)</f>
       </c>
       <c r="U60" t="str">
-        <f>=(B60*1000000)-(C60*10000)+(D60*100)+(E60*1)-(F60*0.01)</f>
+        <f>(B60*1000000)-(C60*10000)+(D60*100)+(E60*1)-(F60*0.01)</f>
       </c>
       <c r="AC60" t="str">
-        <f>=(J60*1000000)-(K60*10000)+(L60*100)+(M60*1)-(N60*0.01)</f>
+        <f>(J60*1000000)-(K60*10000)+(L60*100)+(M60*1)-(N60*0.01)</f>
       </c>
     </row>
     <row r="61">
@@ -7900,10 +7900,10 @@
         <f>RANK(AC61,$AC$60:$AC$62)+COUNTIF($AC$59:AC60,AC61)</f>
       </c>
       <c r="U61" t="str">
-        <f>=(B61*1000000)-(C61*10000)+(D61*100)+(E61*1)-(F61*0.01)</f>
+        <f>(B61*1000000)-(C61*10000)+(D61*100)+(E61*1)-(F61*0.01)</f>
       </c>
       <c r="AC61" t="str">
-        <f>=(J61*1000000)-(K61*10000)+(L61*100)+(M61*1)-(N61*0.01)</f>
+        <f>(J61*1000000)-(K61*10000)+(L61*100)+(M61*1)-(N61*0.01)</f>
       </c>
     </row>
     <row r="62">
@@ -7950,10 +7950,10 @@
         <f>RANK(AC62,$AC$60:$AC$62)+COUNTIF($AC$59:AC61,AC62)</f>
       </c>
       <c r="U62" t="str">
-        <f>=(B62*1000000)-(C62*10000)+(D62*100)+(E62*1)-(F62*0.01)</f>
+        <f>(B62*1000000)-(C62*10000)+(D62*100)+(E62*1)-(F62*0.01)</f>
       </c>
       <c r="AC62" t="str">
-        <f>=(J62*1000000)-(K62*10000)+(L62*100)+(M62*1)-(N62*0.01)</f>
+        <f>(J62*1000000)-(K62*10000)+(L62*100)+(M62*1)-(N62*0.01)</f>
       </c>
     </row>
     <row r="65">
@@ -8208,10 +8208,10 @@
         <f>RANK(AC77,$AC$77:$AC$79)+COUNTIF($AC$76:AC76,AC77)</f>
       </c>
       <c r="U77" t="str">
-        <f>=(B77*1000000)-(C77*10000)+(D77*100)+(E77*1)-(F77*0.01)</f>
+        <f>(B77*1000000)-(C77*10000)+(D77*100)+(E77*1)-(F77*0.01)</f>
       </c>
       <c r="AC77" t="str">
-        <f>=(J77*1000000)-(K77*10000)+(L77*100)+(M77*1)-(N77*0.01)</f>
+        <f>(J77*1000000)-(K77*10000)+(L77*100)+(M77*1)-(N77*0.01)</f>
       </c>
     </row>
     <row r="78">
@@ -8258,10 +8258,10 @@
         <f>RANK(AC78,$AC$77:$AC$79)+COUNTIF($AC$76:AC77,AC78)</f>
       </c>
       <c r="U78" t="str">
-        <f>=(B78*1000000)-(C78*10000)+(D78*100)+(E78*1)-(F78*0.01)</f>
+        <f>(B78*1000000)-(C78*10000)+(D78*100)+(E78*1)-(F78*0.01)</f>
       </c>
       <c r="AC78" t="str">
-        <f>=(J78*1000000)-(K78*10000)+(L78*100)+(M78*1)-(N78*0.01)</f>
+        <f>(J78*1000000)-(K78*10000)+(L78*100)+(M78*1)-(N78*0.01)</f>
       </c>
     </row>
     <row r="79">
@@ -8308,10 +8308,10 @@
         <f>RANK(AC79,$AC$77:$AC$79)+COUNTIF($AC$76:AC78,AC79)</f>
       </c>
       <c r="U79" t="str">
-        <f>=(B79*1000000)-(C79*10000)+(D79*100)+(E79*1)-(F79*0.01)</f>
+        <f>(B79*1000000)-(C79*10000)+(D79*100)+(E79*1)-(F79*0.01)</f>
       </c>
       <c r="AC79" t="str">
-        <f>=(J79*1000000)-(K79*10000)+(L79*100)+(M79*1)-(N79*0.01)</f>
+        <f>(J79*1000000)-(K79*10000)+(L79*100)+(M79*1)-(N79*0.01)</f>
       </c>
     </row>
     <row r="82">
@@ -8566,10 +8566,10 @@
         <f>RANK(AC94,$AC$94:$AC$96)+COUNTIF($AC$93:AC93,AC94)</f>
       </c>
       <c r="U94" t="str">
-        <f>=(B94*1000000)-(C94*10000)+(D94*100)+(E94*1)-(F94*0.01)</f>
+        <f>(B94*1000000)-(C94*10000)+(D94*100)+(E94*1)-(F94*0.01)</f>
       </c>
       <c r="AC94" t="str">
-        <f>=(J94*1000000)-(K94*10000)+(L94*100)+(M94*1)-(N94*0.01)</f>
+        <f>(J94*1000000)-(K94*10000)+(L94*100)+(M94*1)-(N94*0.01)</f>
       </c>
     </row>
     <row r="95">
@@ -8616,10 +8616,10 @@
         <f>RANK(AC95,$AC$94:$AC$96)+COUNTIF($AC$93:AC94,AC95)</f>
       </c>
       <c r="U95" t="str">
-        <f>=(B95*1000000)-(C95*10000)+(D95*100)+(E95*1)-(F95*0.01)</f>
+        <f>(B95*1000000)-(C95*10000)+(D95*100)+(E95*1)-(F95*0.01)</f>
       </c>
       <c r="AC95" t="str">
-        <f>=(J95*1000000)-(K95*10000)+(L95*100)+(M95*1)-(N95*0.01)</f>
+        <f>(J95*1000000)-(K95*10000)+(L95*100)+(M95*1)-(N95*0.01)</f>
       </c>
     </row>
     <row r="96">
@@ -8666,10 +8666,10 @@
         <f>RANK(AC96,$AC$94:$AC$96)+COUNTIF($AC$93:AC95,AC96)</f>
       </c>
       <c r="U96" t="str">
-        <f>=(B96*1000000)-(C96*10000)+(D96*100)+(E96*1)-(F96*0.01)</f>
+        <f>(B96*1000000)-(C96*10000)+(D96*100)+(E96*1)-(F96*0.01)</f>
       </c>
       <c r="AC96" t="str">
-        <f>=(J96*1000000)-(K96*10000)+(L96*100)+(M96*1)-(N96*0.01)</f>
+        <f>(J96*1000000)-(K96*10000)+(L96*100)+(M96*1)-(N96*0.01)</f>
       </c>
     </row>
     <row r="99">
@@ -8924,10 +8924,10 @@
         <f>RANK(AC111,$AC$111:$AC$113)+COUNTIF($AC$110:AC110,AC111)</f>
       </c>
       <c r="U111" t="str">
-        <f>=(B111*1000000)-(C111*10000)+(D111*100)+(E111*1)-(F111*0.01)</f>
+        <f>(B111*1000000)-(C111*10000)+(D111*100)+(E111*1)-(F111*0.01)</f>
       </c>
       <c r="AC111" t="str">
-        <f>=(J111*1000000)-(K111*10000)+(L111*100)+(M111*1)-(N111*0.01)</f>
+        <f>(J111*1000000)-(K111*10000)+(L111*100)+(M111*1)-(N111*0.01)</f>
       </c>
     </row>
     <row r="112">
@@ -8974,10 +8974,10 @@
         <f>RANK(AC112,$AC$111:$AC$113)+COUNTIF($AC$110:AC111,AC112)</f>
       </c>
       <c r="U112" t="str">
-        <f>=(B112*1000000)-(C112*10000)+(D112*100)+(E112*1)-(F112*0.01)</f>
+        <f>(B112*1000000)-(C112*10000)+(D112*100)+(E112*1)-(F112*0.01)</f>
       </c>
       <c r="AC112" t="str">
-        <f>=(J112*1000000)-(K112*10000)+(L112*100)+(M112*1)-(N112*0.01)</f>
+        <f>(J112*1000000)-(K112*10000)+(L112*100)+(M112*1)-(N112*0.01)</f>
       </c>
     </row>
     <row r="113">
@@ -9024,10 +9024,10 @@
         <f>RANK(AC113,$AC$111:$AC$113)+COUNTIF($AC$110:AC112,AC113)</f>
       </c>
       <c r="U113" t="str">
-        <f>=(B113*1000000)-(C113*10000)+(D113*100)+(E113*1)-(F113*0.01)</f>
+        <f>(B113*1000000)-(C113*10000)+(D113*100)+(E113*1)-(F113*0.01)</f>
       </c>
       <c r="AC113" t="str">
-        <f>=(J113*1000000)-(K113*10000)+(L113*100)+(M113*1)-(N113*0.01)</f>
+        <f>(J113*1000000)-(K113*10000)+(L113*100)+(M113*1)-(N113*0.01)</f>
       </c>
     </row>
     <row r="116">
@@ -9282,10 +9282,10 @@
         <f>RANK(AC128,$AC$128:$AC$130)+COUNTIF($AC$127:AC127,AC128)</f>
       </c>
       <c r="U128" t="str">
-        <f>=(B128*1000000)-(C128*10000)+(D128*100)+(E128*1)-(F128*0.01)</f>
+        <f>(B128*1000000)-(C128*10000)+(D128*100)+(E128*1)-(F128*0.01)</f>
       </c>
       <c r="AC128" t="str">
-        <f>=(J128*1000000)-(K128*10000)+(L128*100)+(M128*1)-(N128*0.01)</f>
+        <f>(J128*1000000)-(K128*10000)+(L128*100)+(M128*1)-(N128*0.01)</f>
       </c>
     </row>
     <row r="129">
@@ -9332,10 +9332,10 @@
         <f>RANK(AC129,$AC$128:$AC$130)+COUNTIF($AC$127:AC128,AC129)</f>
       </c>
       <c r="U129" t="str">
-        <f>=(B129*1000000)-(C129*10000)+(D129*100)+(E129*1)-(F129*0.01)</f>
+        <f>(B129*1000000)-(C129*10000)+(D129*100)+(E129*1)-(F129*0.01)</f>
       </c>
       <c r="AC129" t="str">
-        <f>=(J129*1000000)-(K129*10000)+(L129*100)+(M129*1)-(N129*0.01)</f>
+        <f>(J129*1000000)-(K129*10000)+(L129*100)+(M129*1)-(N129*0.01)</f>
       </c>
     </row>
     <row r="130">
@@ -9382,10 +9382,10 @@
         <f>RANK(AC130,$AC$128:$AC$130)+COUNTIF($AC$127:AC129,AC130)</f>
       </c>
       <c r="U130" t="str">
-        <f>=(B130*1000000)-(C130*10000)+(D130*100)+(E130*1)-(F130*0.01)</f>
+        <f>(B130*1000000)-(C130*10000)+(D130*100)+(E130*1)-(F130*0.01)</f>
       </c>
       <c r="AC130" t="str">
-        <f>=(J130*1000000)-(K130*10000)+(L130*100)+(M130*1)-(N130*0.01)</f>
+        <f>(J130*1000000)-(K130*10000)+(L130*100)+(M130*1)-(N130*0.01)</f>
       </c>
     </row>
     <row r="133">
@@ -9640,10 +9640,10 @@
         <f>RANK(AC145,$AC$145:$AC$147)+COUNTIF($AC$144:AC144,AC145)</f>
       </c>
       <c r="U145" t="str">
-        <f>=(B145*1000000)-(C145*10000)+(D145*100)+(E145*1)-(F145*0.01)</f>
+        <f>(B145*1000000)-(C145*10000)+(D145*100)+(E145*1)-(F145*0.01)</f>
       </c>
       <c r="AC145" t="str">
-        <f>=(J145*1000000)-(K145*10000)+(L145*100)+(M145*1)-(N145*0.01)</f>
+        <f>(J145*1000000)-(K145*10000)+(L145*100)+(M145*1)-(N145*0.01)</f>
       </c>
     </row>
     <row r="146">
@@ -9690,10 +9690,10 @@
         <f>RANK(AC146,$AC$145:$AC$147)+COUNTIF($AC$144:AC145,AC146)</f>
       </c>
       <c r="U146" t="str">
-        <f>=(B146*1000000)-(C146*10000)+(D146*100)+(E146*1)-(F146*0.01)</f>
+        <f>(B146*1000000)-(C146*10000)+(D146*100)+(E146*1)-(F146*0.01)</f>
       </c>
       <c r="AC146" t="str">
-        <f>=(J146*1000000)-(K146*10000)+(L146*100)+(M146*1)-(N146*0.01)</f>
+        <f>(J146*1000000)-(K146*10000)+(L146*100)+(M146*1)-(N146*0.01)</f>
       </c>
     </row>
     <row r="147">
@@ -9740,10 +9740,10 @@
         <f>RANK(AC147,$AC$145:$AC$147)+COUNTIF($AC$144:AC146,AC147)</f>
       </c>
       <c r="U147" t="str">
-        <f>=(B147*1000000)-(C147*10000)+(D147*100)+(E147*1)-(F147*0.01)</f>
+        <f>(B147*1000000)-(C147*10000)+(D147*100)+(E147*1)-(F147*0.01)</f>
       </c>
       <c r="AC147" t="str">
-        <f>=(J147*1000000)-(K147*10000)+(L147*100)+(M147*1)-(N147*0.01)</f>
+        <f>(J147*1000000)-(K147*10000)+(L147*100)+(M147*1)-(N147*0.01)</f>
       </c>
     </row>
     <row r="150">
@@ -9998,10 +9998,10 @@
         <f>RANK(AC162,$AC$162:$AC$164)+COUNTIF($AC$161:AC161,AC162)</f>
       </c>
       <c r="U162" t="str">
-        <f>=(B162*1000000)-(C162*10000)+(D162*100)+(E162*1)-(F162*0.01)</f>
+        <f>(B162*1000000)-(C162*10000)+(D162*100)+(E162*1)-(F162*0.01)</f>
       </c>
       <c r="AC162" t="str">
-        <f>=(J162*1000000)-(K162*10000)+(L162*100)+(M162*1)-(N162*0.01)</f>
+        <f>(J162*1000000)-(K162*10000)+(L162*100)+(M162*1)-(N162*0.01)</f>
       </c>
     </row>
     <row r="163">
@@ -10048,10 +10048,10 @@
         <f>RANK(AC163,$AC$162:$AC$164)+COUNTIF($AC$161:AC162,AC163)</f>
       </c>
       <c r="U163" t="str">
-        <f>=(B163*1000000)-(C163*10000)+(D163*100)+(E163*1)-(F163*0.01)</f>
+        <f>(B163*1000000)-(C163*10000)+(D163*100)+(E163*1)-(F163*0.01)</f>
       </c>
       <c r="AC163" t="str">
-        <f>=(J163*1000000)-(K163*10000)+(L163*100)+(M163*1)-(N163*0.01)</f>
+        <f>(J163*1000000)-(K163*10000)+(L163*100)+(M163*1)-(N163*0.01)</f>
       </c>
     </row>
     <row r="164">
@@ -10098,10 +10098,10 @@
         <f>RANK(AC164,$AC$162:$AC$164)+COUNTIF($AC$161:AC163,AC164)</f>
       </c>
       <c r="U164" t="str">
-        <f>=(B164*1000000)-(C164*10000)+(D164*100)+(E164*1)-(F164*0.01)</f>
+        <f>(B164*1000000)-(C164*10000)+(D164*100)+(E164*1)-(F164*0.01)</f>
       </c>
       <c r="AC164" t="str">
-        <f>=(J164*1000000)-(K164*10000)+(L164*100)+(M164*1)-(N164*0.01)</f>
+        <f>(J164*1000000)-(K164*10000)+(L164*100)+(M164*1)-(N164*0.01)</f>
       </c>
     </row>
     <row r="167">
@@ -10356,10 +10356,10 @@
         <f>RANK(AC179,$AC$179:$AC$181)+COUNTIF($AC$178:AC178,AC179)</f>
       </c>
       <c r="U179" t="str">
-        <f>=(B179*1000000)-(C179*10000)+(D179*100)+(E179*1)-(F179*0.01)</f>
+        <f>(B179*1000000)-(C179*10000)+(D179*100)+(E179*1)-(F179*0.01)</f>
       </c>
       <c r="AC179" t="str">
-        <f>=(J179*1000000)-(K179*10000)+(L179*100)+(M179*1)-(N179*0.01)</f>
+        <f>(J179*1000000)-(K179*10000)+(L179*100)+(M179*1)-(N179*0.01)</f>
       </c>
     </row>
     <row r="180">
@@ -10406,10 +10406,10 @@
         <f>RANK(AC180,$AC$179:$AC$181)+COUNTIF($AC$178:AC179,AC180)</f>
       </c>
       <c r="U180" t="str">
-        <f>=(B180*1000000)-(C180*10000)+(D180*100)+(E180*1)-(F180*0.01)</f>
+        <f>(B180*1000000)-(C180*10000)+(D180*100)+(E180*1)-(F180*0.01)</f>
       </c>
       <c r="AC180" t="str">
-        <f>=(J180*1000000)-(K180*10000)+(L180*100)+(M180*1)-(N180*0.01)</f>
+        <f>(J180*1000000)-(K180*10000)+(L180*100)+(M180*1)-(N180*0.01)</f>
       </c>
     </row>
     <row r="181">
@@ -10456,10 +10456,10 @@
         <f>RANK(AC181,$AC$179:$AC$181)+COUNTIF($AC$178:AC180,AC181)</f>
       </c>
       <c r="U181" t="str">
-        <f>=(B181*1000000)-(C181*10000)+(D181*100)+(E181*1)-(F181*0.01)</f>
+        <f>(B181*1000000)-(C181*10000)+(D181*100)+(E181*1)-(F181*0.01)</f>
       </c>
       <c r="AC181" t="str">
-        <f>=(J181*1000000)-(K181*10000)+(L181*100)+(M181*1)-(N181*0.01)</f>
+        <f>(J181*1000000)-(K181*10000)+(L181*100)+(M181*1)-(N181*0.01)</f>
       </c>
     </row>
     <row r="184">
@@ -10714,10 +10714,10 @@
         <f>RANK(AC196,$AC$196:$AC$198)+COUNTIF($AC$195:AC195,AC196)</f>
       </c>
       <c r="U196" t="str">
-        <f>=(B196*1000000)-(C196*10000)+(D196*100)+(E196*1)-(F196*0.01)</f>
+        <f>(B196*1000000)-(C196*10000)+(D196*100)+(E196*1)-(F196*0.01)</f>
       </c>
       <c r="AC196" t="str">
-        <f>=(J196*1000000)-(K196*10000)+(L196*100)+(M196*1)-(N196*0.01)</f>
+        <f>(J196*1000000)-(K196*10000)+(L196*100)+(M196*1)-(N196*0.01)</f>
       </c>
     </row>
     <row r="197">
@@ -10764,10 +10764,10 @@
         <f>RANK(AC197,$AC$196:$AC$198)+COUNTIF($AC$195:AC196,AC197)</f>
       </c>
       <c r="U197" t="str">
-        <f>=(B197*1000000)-(C197*10000)+(D197*100)+(E197*1)-(F197*0.01)</f>
+        <f>(B197*1000000)-(C197*10000)+(D197*100)+(E197*1)-(F197*0.01)</f>
       </c>
       <c r="AC197" t="str">
-        <f>=(J197*1000000)-(K197*10000)+(L197*100)+(M197*1)-(N197*0.01)</f>
+        <f>(J197*1000000)-(K197*10000)+(L197*100)+(M197*1)-(N197*0.01)</f>
       </c>
     </row>
     <row r="198">
@@ -10814,10 +10814,10 @@
         <f>RANK(AC198,$AC$196:$AC$198)+COUNTIF($AC$195:AC197,AC198)</f>
       </c>
       <c r="U198" t="str">
-        <f>=(B198*1000000)-(C198*10000)+(D198*100)+(E198*1)-(F198*0.01)</f>
+        <f>(B198*1000000)-(C198*10000)+(D198*100)+(E198*1)-(F198*0.01)</f>
       </c>
       <c r="AC198" t="str">
-        <f>=(J198*1000000)-(K198*10000)+(L198*100)+(M198*1)-(N198*0.01)</f>
+        <f>(J198*1000000)-(K198*10000)+(L198*100)+(M198*1)-(N198*0.01)</f>
       </c>
     </row>
     <row r="201">
@@ -11072,10 +11072,10 @@
         <f>RANK(AC213,$AC$213:$AC$215)+COUNTIF($AC$212:AC212,AC213)</f>
       </c>
       <c r="U213" t="str">
-        <f>=(B213*1000000)-(C213*10000)+(D213*100)+(E213*1)-(F213*0.01)</f>
+        <f>(B213*1000000)-(C213*10000)+(D213*100)+(E213*1)-(F213*0.01)</f>
       </c>
       <c r="AC213" t="str">
-        <f>=(J213*1000000)-(K213*10000)+(L213*100)+(M213*1)-(N213*0.01)</f>
+        <f>(J213*1000000)-(K213*10000)+(L213*100)+(M213*1)-(N213*0.01)</f>
       </c>
     </row>
     <row r="214">
@@ -11122,10 +11122,10 @@
         <f>RANK(AC214,$AC$213:$AC$215)+COUNTIF($AC$212:AC213,AC214)</f>
       </c>
       <c r="U214" t="str">
-        <f>=(B214*1000000)-(C214*10000)+(D214*100)+(E214*1)-(F214*0.01)</f>
+        <f>(B214*1000000)-(C214*10000)+(D214*100)+(E214*1)-(F214*0.01)</f>
       </c>
       <c r="AC214" t="str">
-        <f>=(J214*1000000)-(K214*10000)+(L214*100)+(M214*1)-(N214*0.01)</f>
+        <f>(J214*1000000)-(K214*10000)+(L214*100)+(M214*1)-(N214*0.01)</f>
       </c>
     </row>
     <row r="215">
@@ -11172,10 +11172,10 @@
         <f>RANK(AC215,$AC$213:$AC$215)+COUNTIF($AC$212:AC214,AC215)</f>
       </c>
       <c r="U215" t="str">
-        <f>=(B215*1000000)-(C215*10000)+(D215*100)+(E215*1)-(F215*0.01)</f>
+        <f>(B215*1000000)-(C215*10000)+(D215*100)+(E215*1)-(F215*0.01)</f>
       </c>
       <c r="AC215" t="str">
-        <f>=(J215*1000000)-(K215*10000)+(L215*100)+(M215*1)-(N215*0.01)</f>
+        <f>(J215*1000000)-(K215*10000)+(L215*100)+(M215*1)-(N215*0.01)</f>
       </c>
     </row>
     <row r="218">
@@ -11430,10 +11430,10 @@
         <f>RANK(AC230,$AC$230:$AC$232)+COUNTIF($AC$229:AC229,AC230)</f>
       </c>
       <c r="U230" t="str">
-        <f>=(B230*1000000)-(C230*10000)+(D230*100)+(E230*1)-(F230*0.01)</f>
+        <f>(B230*1000000)-(C230*10000)+(D230*100)+(E230*1)-(F230*0.01)</f>
       </c>
       <c r="AC230" t="str">
-        <f>=(J230*1000000)-(K230*10000)+(L230*100)+(M230*1)-(N230*0.01)</f>
+        <f>(J230*1000000)-(K230*10000)+(L230*100)+(M230*1)-(N230*0.01)</f>
       </c>
     </row>
     <row r="231">
@@ -11480,10 +11480,10 @@
         <f>RANK(AC231,$AC$230:$AC$232)+COUNTIF($AC$229:AC230,AC231)</f>
       </c>
       <c r="U231" t="str">
-        <f>=(B231*1000000)-(C231*10000)+(D231*100)+(E231*1)-(F231*0.01)</f>
+        <f>(B231*1000000)-(C231*10000)+(D231*100)+(E231*1)-(F231*0.01)</f>
       </c>
       <c r="AC231" t="str">
-        <f>=(J231*1000000)-(K231*10000)+(L231*100)+(M231*1)-(N231*0.01)</f>
+        <f>(J231*1000000)-(K231*10000)+(L231*100)+(M231*1)-(N231*0.01)</f>
       </c>
     </row>
     <row r="232">
@@ -11530,10 +11530,10 @@
         <f>RANK(AC232,$AC$230:$AC$232)+COUNTIF($AC$229:AC231,AC232)</f>
       </c>
       <c r="U232" t="str">
-        <f>=(B232*1000000)-(C232*10000)+(D232*100)+(E232*1)-(F232*0.01)</f>
+        <f>(B232*1000000)-(C232*10000)+(D232*100)+(E232*1)-(F232*0.01)</f>
       </c>
       <c r="AC232" t="str">
-        <f>=(J232*1000000)-(K232*10000)+(L232*100)+(M232*1)-(N232*0.01)</f>
+        <f>(J232*1000000)-(K232*10000)+(L232*100)+(M232*1)-(N232*0.01)</f>
       </c>
     </row>
     <row r="235">
@@ -11766,10 +11766,10 @@
         <f>RANK(AC247,$AC$247:$AC$248)+COUNTIF($AC$246:AC246,AC247)</f>
       </c>
       <c r="U247" t="str">
-        <f>=(B247*1000000)-(C247*10000)+(D247*100)+(E247*1)-(F247*0.01)</f>
+        <f>(B247*1000000)-(C247*10000)+(D247*100)+(E247*1)-(F247*0.01)</f>
       </c>
       <c r="AC247" t="str">
-        <f>=(J247*1000000)-(K247*10000)+(L247*100)+(M247*1)-(N247*0.01)</f>
+        <f>(J247*1000000)-(K247*10000)+(L247*100)+(M247*1)-(N247*0.01)</f>
       </c>
     </row>
     <row r="248">
@@ -11816,10 +11816,10 @@
         <f>RANK(AC248,$AC$247:$AC$248)+COUNTIF($AC$246:AC247,AC248)</f>
       </c>
       <c r="U248" t="str">
-        <f>=(B248*1000000)-(C248*10000)+(D248*100)+(E248*1)-(F248*0.01)</f>
+        <f>(B248*1000000)-(C248*10000)+(D248*100)+(E248*1)-(F248*0.01)</f>
       </c>
       <c r="AC248" t="str">
-        <f>=(J248*1000000)-(K248*10000)+(L248*100)+(M248*1)-(N248*0.01)</f>
+        <f>(J248*1000000)-(K248*10000)+(L248*100)+(M248*1)-(N248*0.01)</f>
       </c>
     </row>
     <row r="249">
@@ -11845,7 +11845,7 @@
         <f>RANK(U249,$U$247:$U$249)+COUNTIF($U$246:U248,U249)</f>
       </c>
       <c r="U249" t="str">
-        <f>=(B249*1000000)-(C249*10000)+(D249*100)+(E249*1)-(F249*0.01)</f>
+        <f>(B249*1000000)-(C249*10000)+(D249*100)+(E249*1)-(F249*0.01)</f>
       </c>
     </row>
     <row r="251">
@@ -11977,7 +11977,7 @@
         <f>RANK(U262,$U$262:$U$263)+COUNTIF($U$261:U261,U262)</f>
       </c>
       <c r="U262" t="str">
-        <f>=(B262*1000000)-(C262*10000)+(D262*100)+(E262*1)-(F262*0.01)</f>
+        <f>(B262*1000000)-(C262*10000)+(D262*100)+(E262*1)-(F262*0.01)</f>
       </c>
     </row>
     <row r="263">
@@ -12003,7 +12003,7 @@
         <f>RANK(U263,$U$262:$U$263)+COUNTIF($U$261:U262,U263)</f>
       </c>
       <c r="U263" t="str">
-        <f>=(B263*1000000)-(C263*10000)+(D263*100)+(E263*1)-(F263*0.01)</f>
+        <f>(B263*1000000)-(C263*10000)+(D263*100)+(E263*1)-(F263*0.01)</f>
       </c>
     </row>
     <row r="266">

</xml_diff>

<commit_message>
fix(tags): fix QR deep-link URL and finalize tag layout
- Change QR URL path from /viewer.html to / so the SPA doesn't
  rewrite the URL and strip the ?playerNumber= query string before
  resolveDeepLink can process it
- Tag layout: 250pt Calibri Bold, column width 110, two tags per A4
  page (one 409pt row each), QR at OffsetX=57 OffsetY=242 (left of
  number, vertically aligned with its centre)
- Update qr_test.go expected URLs accordingly
- Regenerate example XLSX files

Closes mp-yin4

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pools-example-large-max-size.xlsx
+++ b/pools-example-large-max-size.xlsx
@@ -1367,7 +1367,7 @@
       <family val="2"/>
       <b val="1"/>
       <color/>
-      <sz val="150"/>
+      <sz val="200"/>
     </font>
   </fonts>
   <fills count="6">
@@ -4730,912 +4730,912 @@
     <col customWidth="true" max="1" min="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" ht="390" customHeight="true">
+    <row r="1" ht="409" customHeight="true">
       <c r="A1" s="30" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="2" ht="390" customHeight="true">
+    <row r="2" ht="409" customHeight="true">
       <c r="A2" s="30" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="3" ht="390" customHeight="true">
+    <row r="3" ht="409" customHeight="true">
       <c r="A3" s="30" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="4" ht="390" customHeight="true">
+    <row r="4" ht="409" customHeight="true">
       <c r="A4" s="30" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="5" ht="390" customHeight="true">
+    <row r="5" ht="409" customHeight="true">
       <c r="A5" s="30" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="6" ht="390" customHeight="true">
+    <row r="6" ht="409" customHeight="true">
       <c r="A6" s="30" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="7" ht="390" customHeight="true">
+    <row r="7" ht="409" customHeight="true">
       <c r="A7" s="30" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="8" ht="390" customHeight="true">
+    <row r="8" ht="409" customHeight="true">
       <c r="A8" s="30" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="9" ht="390" customHeight="true">
+    <row r="9" ht="409" customHeight="true">
       <c r="A9" s="30" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="10" ht="390" customHeight="true">
+    <row r="10" ht="409" customHeight="true">
       <c r="A10" s="30" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="11" ht="390" customHeight="true">
+    <row r="11" ht="409" customHeight="true">
       <c r="A11" s="30" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="12" ht="390" customHeight="true">
+    <row r="12" ht="409" customHeight="true">
       <c r="A12" s="30" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="13" ht="390" customHeight="true">
+    <row r="13" ht="409" customHeight="true">
       <c r="A13" s="30" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="14" ht="390" customHeight="true">
+    <row r="14" ht="409" customHeight="true">
       <c r="A14" s="30" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="15" ht="390" customHeight="true">
+    <row r="15" ht="409" customHeight="true">
       <c r="A15" s="30" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="16" ht="390" customHeight="true">
+    <row r="16" ht="409" customHeight="true">
       <c r="A16" s="30" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="17" ht="390" customHeight="true">
+    <row r="17" ht="409" customHeight="true">
       <c r="A17" s="30" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="18" ht="390" customHeight="true">
+    <row r="18" ht="409" customHeight="true">
       <c r="A18" s="30" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="19" ht="390" customHeight="true">
+    <row r="19" ht="409" customHeight="true">
       <c r="A19" s="30" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="20" ht="390" customHeight="true">
+    <row r="20" ht="409" customHeight="true">
       <c r="A20" s="30" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="21" ht="390" customHeight="true">
+    <row r="21" ht="409" customHeight="true">
       <c r="A21" s="30" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="22" ht="390" customHeight="true">
+    <row r="22" ht="409" customHeight="true">
       <c r="A22" s="30" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="23" ht="390" customHeight="true">
+    <row r="23" ht="409" customHeight="true">
       <c r="A23" s="30" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="24" ht="390" customHeight="true">
+    <row r="24" ht="409" customHeight="true">
       <c r="A24" s="30" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="25" ht="390" customHeight="true">
+    <row r="25" ht="409" customHeight="true">
       <c r="A25" s="30" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="26" ht="390" customHeight="true">
+    <row r="26" ht="409" customHeight="true">
       <c r="A26" s="30" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="27" ht="390" customHeight="true">
+    <row r="27" ht="409" customHeight="true">
       <c r="A27" s="30" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="28" ht="390" customHeight="true">
+    <row r="28" ht="409" customHeight="true">
       <c r="A28" s="30" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="29" ht="390" customHeight="true">
+    <row r="29" ht="409" customHeight="true">
       <c r="A29" s="30" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="30" ht="390" customHeight="true">
+    <row r="30" ht="409" customHeight="true">
       <c r="A30" s="30" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="31" ht="390" customHeight="true">
+    <row r="31" ht="409" customHeight="true">
       <c r="A31" s="30" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="32" ht="390" customHeight="true">
+    <row r="32" ht="409" customHeight="true">
       <c r="A32" s="30" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="33" ht="390" customHeight="true">
+    <row r="33" ht="409" customHeight="true">
       <c r="A33" s="30" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="34" ht="390" customHeight="true">
+    <row r="34" ht="409" customHeight="true">
       <c r="A34" s="30" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="35" ht="390" customHeight="true">
+    <row r="35" ht="409" customHeight="true">
       <c r="A35" s="30" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="36" ht="390" customHeight="true">
+    <row r="36" ht="409" customHeight="true">
       <c r="A36" s="30" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="37" ht="390" customHeight="true">
+    <row r="37" ht="409" customHeight="true">
       <c r="A37" s="30" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="38" ht="390" customHeight="true">
+    <row r="38" ht="409" customHeight="true">
       <c r="A38" s="30" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="39" ht="390" customHeight="true">
+    <row r="39" ht="409" customHeight="true">
       <c r="A39" s="30" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="40" ht="390" customHeight="true">
+    <row r="40" ht="409" customHeight="true">
       <c r="A40" s="30" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="41" ht="390" customHeight="true">
+    <row r="41" ht="409" customHeight="true">
       <c r="A41" s="30" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="42" ht="390" customHeight="true">
+    <row r="42" ht="409" customHeight="true">
       <c r="A42" s="30" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="43" ht="390" customHeight="true">
+    <row r="43" ht="409" customHeight="true">
       <c r="A43" s="30" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="44" ht="390" customHeight="true">
+    <row r="44" ht="409" customHeight="true">
       <c r="A44" s="30" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="45" ht="390" customHeight="true">
+    <row r="45" ht="409" customHeight="true">
       <c r="A45" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="46" ht="390" customHeight="true">
+    <row r="46" ht="409" customHeight="true">
       <c r="A46" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="47" ht="390" customHeight="true">
+    <row r="47" ht="409" customHeight="true">
       <c r="A47" s="30" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="48" ht="390" customHeight="true">
+    <row r="48" ht="409" customHeight="true">
       <c r="A48" s="30" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="49" ht="390" customHeight="true">
+    <row r="49" ht="409" customHeight="true">
       <c r="A49" s="30" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="50" ht="390" customHeight="true">
+    <row r="50" ht="409" customHeight="true">
       <c r="A50" s="30" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="51" ht="390" customHeight="true">
+    <row r="51" ht="409" customHeight="true">
       <c r="A51" s="30" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="52" ht="390" customHeight="true">
+    <row r="52" ht="409" customHeight="true">
       <c r="A52" s="30" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="53" ht="390" customHeight="true">
+    <row r="53" ht="409" customHeight="true">
       <c r="A53" s="30" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="54" ht="390" customHeight="true">
+    <row r="54" ht="409" customHeight="true">
       <c r="A54" s="30" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="55" ht="390" customHeight="true">
+    <row r="55" ht="409" customHeight="true">
       <c r="A55" s="30" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="56" ht="390" customHeight="true">
+    <row r="56" ht="409" customHeight="true">
       <c r="A56" s="30" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="57" ht="390" customHeight="true">
+    <row r="57" ht="409" customHeight="true">
       <c r="A57" s="30" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="58" ht="390" customHeight="true">
+    <row r="58" ht="409" customHeight="true">
       <c r="A58" s="30" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="59" ht="390" customHeight="true">
+    <row r="59" ht="409" customHeight="true">
       <c r="A59" s="30" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="60" ht="390" customHeight="true">
+    <row r="60" ht="409" customHeight="true">
       <c r="A60" s="30" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="61" ht="390" customHeight="true">
+    <row r="61" ht="409" customHeight="true">
       <c r="A61" s="30" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="62" ht="390" customHeight="true">
+    <row r="62" ht="409" customHeight="true">
       <c r="A62" s="30" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="63" ht="390" customHeight="true">
+    <row r="63" ht="409" customHeight="true">
       <c r="A63" s="30" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="64" ht="390" customHeight="true">
+    <row r="64" ht="409" customHeight="true">
       <c r="A64" s="30" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="65" ht="390" customHeight="true">
+    <row r="65" ht="409" customHeight="true">
       <c r="A65" s="30" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="66" ht="390" customHeight="true">
+    <row r="66" ht="409" customHeight="true">
       <c r="A66" s="30" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="67" ht="390" customHeight="true">
+    <row r="67" ht="409" customHeight="true">
       <c r="A67" s="30" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="68" ht="390" customHeight="true">
+    <row r="68" ht="409" customHeight="true">
       <c r="A68" s="30" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="69" ht="390" customHeight="true">
+    <row r="69" ht="409" customHeight="true">
       <c r="A69" s="30" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="70" ht="390" customHeight="true">
+    <row r="70" ht="409" customHeight="true">
       <c r="A70" s="30" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="71" ht="390" customHeight="true">
+    <row r="71" ht="409" customHeight="true">
       <c r="A71" s="30" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="72" ht="390" customHeight="true">
+    <row r="72" ht="409" customHeight="true">
       <c r="A72" s="30" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="73" ht="390" customHeight="true">
+    <row r="73" ht="409" customHeight="true">
       <c r="A73" s="30" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="74" ht="390" customHeight="true">
+    <row r="74" ht="409" customHeight="true">
       <c r="A74" s="30" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="75" ht="390" customHeight="true">
+    <row r="75" ht="409" customHeight="true">
       <c r="A75" s="30" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="76" ht="390" customHeight="true">
+    <row r="76" ht="409" customHeight="true">
       <c r="A76" s="30" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="77" ht="390" customHeight="true">
+    <row r="77" ht="409" customHeight="true">
       <c r="A77" s="30" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="78" ht="390" customHeight="true">
+    <row r="78" ht="409" customHeight="true">
       <c r="A78" s="30" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="79" ht="390" customHeight="true">
+    <row r="79" ht="409" customHeight="true">
       <c r="A79" s="30" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="80" ht="390" customHeight="true">
+    <row r="80" ht="409" customHeight="true">
       <c r="A80" s="30" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="81" ht="390" customHeight="true">
+    <row r="81" ht="409" customHeight="true">
       <c r="A81" s="30" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="82" ht="390" customHeight="true">
+    <row r="82" ht="409" customHeight="true">
       <c r="A82" s="30" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="83" ht="390" customHeight="true">
+    <row r="83" ht="409" customHeight="true">
       <c r="A83" s="30" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="84" ht="390" customHeight="true">
+    <row r="84" ht="409" customHeight="true">
       <c r="A84" s="30" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="85" ht="390" customHeight="true">
+    <row r="85" ht="409" customHeight="true">
       <c r="A85" s="30" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="86" ht="390" customHeight="true">
+    <row r="86" ht="409" customHeight="true">
       <c r="A86" s="30" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="87" ht="390" customHeight="true">
+    <row r="87" ht="409" customHeight="true">
       <c r="A87" s="30" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="88" ht="390" customHeight="true">
+    <row r="88" ht="409" customHeight="true">
       <c r="A88" s="30" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="89" ht="390" customHeight="true">
+    <row r="89" ht="409" customHeight="true">
       <c r="A89" s="30" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="90" ht="390" customHeight="true">
+    <row r="90" ht="409" customHeight="true">
       <c r="A90" s="30" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="91" ht="390" customHeight="true">
+    <row r="91" ht="409" customHeight="true">
       <c r="A91" s="30" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="92" ht="390" customHeight="true">
+    <row r="92" ht="409" customHeight="true">
       <c r="A92" s="30" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="93" ht="390" customHeight="true">
+    <row r="93" ht="409" customHeight="true">
       <c r="A93" s="30" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="94" ht="390" customHeight="true">
+    <row r="94" ht="409" customHeight="true">
       <c r="A94" s="30" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="95" ht="390" customHeight="true">
+    <row r="95" ht="409" customHeight="true">
       <c r="A95" s="30" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="96" ht="390" customHeight="true">
+    <row r="96" ht="409" customHeight="true">
       <c r="A96" s="30" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="97" ht="390" customHeight="true">
+    <row r="97" ht="409" customHeight="true">
       <c r="A97" s="30" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="98" ht="390" customHeight="true">
+    <row r="98" ht="409" customHeight="true">
       <c r="A98" s="30" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="99" ht="390" customHeight="true">
+    <row r="99" ht="409" customHeight="true">
       <c r="A99" s="30" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="100" ht="390" customHeight="true">
+    <row r="100" ht="409" customHeight="true">
       <c r="A100" s="30" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="101" ht="390" customHeight="true">
+    <row r="101" ht="409" customHeight="true">
       <c r="A101" s="30" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="102" ht="390" customHeight="true">
+    <row r="102" ht="409" customHeight="true">
       <c r="A102" s="30" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="103" ht="390" customHeight="true">
+    <row r="103" ht="409" customHeight="true">
       <c r="A103" s="30" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="104" ht="390" customHeight="true">
+    <row r="104" ht="409" customHeight="true">
       <c r="A104" s="30" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="105" ht="390" customHeight="true">
+    <row r="105" ht="409" customHeight="true">
       <c r="A105" s="30" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="106" ht="390" customHeight="true">
+    <row r="106" ht="409" customHeight="true">
       <c r="A106" s="30" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="107" ht="390" customHeight="true">
+    <row r="107" ht="409" customHeight="true">
       <c r="A107" s="30" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="108" ht="390" customHeight="true">
+    <row r="108" ht="409" customHeight="true">
       <c r="A108" s="30" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="109" ht="390" customHeight="true">
+    <row r="109" ht="409" customHeight="true">
       <c r="A109" s="30" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="110" ht="390" customHeight="true">
+    <row r="110" ht="409" customHeight="true">
       <c r="A110" s="30" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="111" ht="390" customHeight="true">
+    <row r="111" ht="409" customHeight="true">
       <c r="A111" s="30" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="112" ht="390" customHeight="true">
+    <row r="112" ht="409" customHeight="true">
       <c r="A112" s="30" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="113" ht="390" customHeight="true">
+    <row r="113" ht="409" customHeight="true">
       <c r="A113" s="30" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="114" ht="390" customHeight="true">
+    <row r="114" ht="409" customHeight="true">
       <c r="A114" s="30" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="115" ht="390" customHeight="true">
+    <row r="115" ht="409" customHeight="true">
       <c r="A115" s="30" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="116" ht="390" customHeight="true">
+    <row r="116" ht="409" customHeight="true">
       <c r="A116" s="30" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="117" ht="390" customHeight="true">
+    <row r="117" ht="409" customHeight="true">
       <c r="A117" s="30" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="118" ht="390" customHeight="true">
+    <row r="118" ht="409" customHeight="true">
       <c r="A118" s="30" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="119" ht="390" customHeight="true">
+    <row r="119" ht="409" customHeight="true">
       <c r="A119" s="30" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="120" ht="390" customHeight="true">
+    <row r="120" ht="409" customHeight="true">
       <c r="A120" s="30" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="121" ht="390" customHeight="true">
+    <row r="121" ht="409" customHeight="true">
       <c r="A121" s="30" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="122" ht="390" customHeight="true">
+    <row r="122" ht="409" customHeight="true">
       <c r="A122" s="30" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="123" ht="390" customHeight="true">
+    <row r="123" ht="409" customHeight="true">
       <c r="A123" s="30" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="124" ht="390" customHeight="true">
+    <row r="124" ht="409" customHeight="true">
       <c r="A124" s="30" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="125" ht="390" customHeight="true">
+    <row r="125" ht="409" customHeight="true">
       <c r="A125" s="30" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="126" ht="390" customHeight="true">
+    <row r="126" ht="409" customHeight="true">
       <c r="A126" s="30" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="127" ht="390" customHeight="true">
+    <row r="127" ht="409" customHeight="true">
       <c r="A127" s="30" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="128" ht="390" customHeight="true">
+    <row r="128" ht="409" customHeight="true">
       <c r="A128" s="30" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="129" ht="390" customHeight="true">
+    <row r="129" ht="409" customHeight="true">
       <c r="A129" s="30" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="130" ht="390" customHeight="true">
+    <row r="130" ht="409" customHeight="true">
       <c r="A130" s="30" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="131" ht="390" customHeight="true">
+    <row r="131" ht="409" customHeight="true">
       <c r="A131" s="30" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="132" ht="390" customHeight="true">
+    <row r="132" ht="409" customHeight="true">
       <c r="A132" s="30" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="133" ht="390" customHeight="true">
+    <row r="133" ht="409" customHeight="true">
       <c r="A133" s="30" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="134" ht="390" customHeight="true">
+    <row r="134" ht="409" customHeight="true">
       <c r="A134" s="30" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="135" ht="390" customHeight="true">
+    <row r="135" ht="409" customHeight="true">
       <c r="A135" s="30" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="136" ht="390" customHeight="true">
+    <row r="136" ht="409" customHeight="true">
       <c r="A136" s="30" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="137" ht="390" customHeight="true">
+    <row r="137" ht="409" customHeight="true">
       <c r="A137" s="30" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="138" ht="390" customHeight="true">
+    <row r="138" ht="409" customHeight="true">
       <c r="A138" s="30" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="139" ht="390" customHeight="true">
+    <row r="139" ht="409" customHeight="true">
       <c r="A139" s="30" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="140" ht="390" customHeight="true">
+    <row r="140" ht="409" customHeight="true">
       <c r="A140" s="30" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="141" ht="390" customHeight="true">
+    <row r="141" ht="409" customHeight="true">
       <c r="A141" s="30" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="142" ht="390" customHeight="true">
+    <row r="142" ht="409" customHeight="true">
       <c r="A142" s="30" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="143" ht="390" customHeight="true">
+    <row r="143" ht="409" customHeight="true">
       <c r="A143" s="30" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="144" ht="390" customHeight="true">
+    <row r="144" ht="409" customHeight="true">
       <c r="A144" s="30" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="145" ht="390" customHeight="true">
+    <row r="145" ht="409" customHeight="true">
       <c r="A145" s="30" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="146" ht="390" customHeight="true">
+    <row r="146" ht="409" customHeight="true">
       <c r="A146" s="30" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="147" ht="390" customHeight="true">
+    <row r="147" ht="409" customHeight="true">
       <c r="A147" s="30" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="148" ht="390" customHeight="true">
+    <row r="148" ht="409" customHeight="true">
       <c r="A148" s="30" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="149" ht="390" customHeight="true">
+    <row r="149" ht="409" customHeight="true">
       <c r="A149" s="30" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="150" ht="390" customHeight="true">
+    <row r="150" ht="409" customHeight="true">
       <c r="A150" s="30" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="151" ht="390" customHeight="true">
+    <row r="151" ht="409" customHeight="true">
       <c r="A151" s="30" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="152" ht="390" customHeight="true">
+    <row r="152" ht="409" customHeight="true">
       <c r="A152" s="30" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="153" ht="390" customHeight="true">
+    <row r="153" ht="409" customHeight="true">
       <c r="A153" s="30" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="154" ht="390" customHeight="true">
+    <row r="154" ht="409" customHeight="true">
       <c r="A154" s="30" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="155" ht="390" customHeight="true">
+    <row r="155" ht="409" customHeight="true">
       <c r="A155" s="30" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="156" ht="390" customHeight="true">
+    <row r="156" ht="409" customHeight="true">
       <c r="A156" s="30" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="157" ht="390" customHeight="true">
+    <row r="157" ht="409" customHeight="true">
       <c r="A157" s="30" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="158" ht="390" customHeight="true">
+    <row r="158" ht="409" customHeight="true">
       <c r="A158" s="30" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="159" ht="390" customHeight="true">
+    <row r="159" ht="409" customHeight="true">
       <c r="A159" s="30" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="160" ht="390" customHeight="true">
+    <row r="160" ht="409" customHeight="true">
       <c r="A160" s="30" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="161" ht="390" customHeight="true">
+    <row r="161" ht="409" customHeight="true">
       <c r="A161" s="30" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="162" ht="390" customHeight="true">
+    <row r="162" ht="409" customHeight="true">
       <c r="A162" s="30" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="163" ht="390" customHeight="true">
+    <row r="163" ht="409" customHeight="true">
       <c r="A163" s="30" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="164" ht="390" customHeight="true">
+    <row r="164" ht="409" customHeight="true">
       <c r="A164" s="30" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="165" ht="390" customHeight="true">
+    <row r="165" ht="409" customHeight="true">
       <c r="A165" s="30" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="166" ht="390" customHeight="true">
+    <row r="166" ht="409" customHeight="true">
       <c r="A166" s="30" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="167" ht="390" customHeight="true">
+    <row r="167" ht="409" customHeight="true">
       <c r="A167" s="30" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="168" ht="390" customHeight="true">
+    <row r="168" ht="409" customHeight="true">
       <c r="A168" s="30" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="169" ht="390" customHeight="true">
+    <row r="169" ht="409" customHeight="true">
       <c r="A169" s="30" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="170" ht="390" customHeight="true">
+    <row r="170" ht="409" customHeight="true">
       <c r="A170" s="30" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="171" ht="390" customHeight="true">
+    <row r="171" ht="409" customHeight="true">
       <c r="A171" s="30" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="172" ht="390" customHeight="true">
+    <row r="172" ht="409" customHeight="true">
       <c r="A172" s="30" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="173" ht="390" customHeight="true">
+    <row r="173" ht="409" customHeight="true">
       <c r="A173" s="30" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="174" ht="390" customHeight="true">
+    <row r="174" ht="409" customHeight="true">
       <c r="A174" s="30" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="175" ht="390" customHeight="true">
+    <row r="175" ht="409" customHeight="true">
       <c r="A175" s="30" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="176" ht="390" customHeight="true">
+    <row r="176" ht="409" customHeight="true">
       <c r="A176" s="30" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="177" ht="390" customHeight="true">
+    <row r="177" ht="409" customHeight="true">
       <c r="A177" s="30" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="178" ht="390" customHeight="true">
+    <row r="178" ht="409" customHeight="true">
       <c r="A178" s="30" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="179" ht="390" customHeight="true">
+    <row r="179" ht="409" customHeight="true">
       <c r="A179" s="30" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="180" ht="390" customHeight="true">
+    <row r="180" ht="409" customHeight="true">
       <c r="A180" s="30" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="181" ht="390" customHeight="true">
+    <row r="181" ht="409" customHeight="true">
       <c r="A181" s="30" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="182" ht="390" customHeight="true">
+    <row r="182" ht="409" customHeight="true">
       <c r="A182" s="30" t="s">
         <v>343</v>
       </c>

</xml_diff>

<commit_message>
feat(mp-hhea): add two-layer API rate limiting and loading spinner
- Global circuit breaker (5000 req/s, burst 10000) prevents total server
  overload. Configurable via API_RATE_LIMIT and API_RATE_LIMIT_BURST env
  vars with > 0 validation and startup logging.
- Per-IP fairness layer (100 req/s, burst 200) prevents a single client
  from exhausting the global budget and starving other users. Zero-config
  with automatic TTL cleanup of idle IP entries (5min idle, 3min sweep).
- Both layers are zero-config with sensible defaults — the operator does
  not need to configure anything for protection to activate.
- LoadingSpinner component with 200ms delay to prevent flicker on fast
  loads. Integrated into app, admin, and viewer entry points.
- Stale CSS comment cleanup for tablet portrait layout.
</commit_message>
<xml_diff>
--- a/pools-example-large-max-size.xlsx
+++ b/pools-example-large-max-size.xlsx
@@ -1367,7 +1367,7 @@
       <family val="2"/>
       <b val="1"/>
       <color/>
-      <sz val="200"/>
+      <sz val="250"/>
     </font>
   </fonts>
   <fills count="6">
@@ -4727,7 +4727,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="90"/>
+    <col customWidth="true" max="1" min="1" width="110"/>
   </cols>
   <sheetData>
     <row r="1" ht="409" customHeight="true">

</xml_diff>